<commit_message>
fetch data from deribit
</commit_message>
<xml_diff>
--- a/table1_timestep_dts.xlsx
+++ b/table1_timestep_dts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\27261\Desktop\3_Courses in PHBS\3_09_AppliedStochasticProcess\Project_sv32_EMC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_3AF1827E134D482EEB75ECF65B5DCE3A874752DE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{818883F2-2ECA-4A42-87C8-594A5906AD45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="279">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="271">
   <si>
     <t>Euler/Milstein scheme</t>
   </si>
@@ -652,45 +652,30 @@
     <t>0.01475 (0.12%)</t>
   </si>
   <si>
-    <t>4.106e+68 (3223301308466970432709825405034145773061746998061010581630537663774720.00%)</t>
-  </si>
-  <si>
     <t>-0.0573 (-0.46%)</t>
   </si>
   <si>
     <t>0.01432 (0.12%)</t>
   </si>
   <si>
-    <t>4.106e+68 (3313703904466378806464151377072601387691560996216091668196808529543168.00%)</t>
-  </si>
-  <si>
     <t>-0.05718 (-0.47%)</t>
   </si>
   <si>
     <t>0.01395 (0.12%)</t>
   </si>
   <si>
-    <t>4.106e+68 (3405477907361264938249467604493313804006482743010814697689290012360704.00%)</t>
-  </si>
-  <si>
     <t>-0.05727 (-0.49%)</t>
   </si>
   <si>
     <t>0.01336 (0.11%)</t>
   </si>
   <si>
-    <t>4.106e+68 (3498510749065141853418263297025261283428080760865694523030412172722176.00%)</t>
-  </si>
-  <si>
     <t>-0.05716 (-0.50%)</t>
   </si>
   <si>
     <t>0.01297 (0.11%)</t>
   </si>
   <si>
-    <t>4.106e+68 (3592897950235740819834831940019451353856068708643917677792140514557952.00%)</t>
-  </si>
-  <si>
     <t>468.6 (3678.98%)</t>
   </si>
   <si>
@@ -700,9 +685,6 @@
     <t>0.02753 (0.22%)</t>
   </si>
   <si>
-    <t>3.057e+21 (24003062986973477076992.00%)</t>
-  </si>
-  <si>
     <t>468.6 (3782.16%)</t>
   </si>
   <si>
@@ -712,9 +694,6 @@
     <t>0.02743 (0.22%)</t>
   </si>
   <si>
-    <t>3.057e+21 (24676266947229916332032.00%)</t>
-  </si>
-  <si>
     <t>468.6 (3886.91%)</t>
   </si>
   <si>
@@ -724,9 +703,6 @@
     <t>0.02739 (0.23%)</t>
   </si>
   <si>
-    <t>3.057e+21 (25359683407945570189312.00%)</t>
-  </si>
-  <si>
     <t>468.6 (3993.10%)</t>
   </si>
   <si>
@@ -736,9 +712,6 @@
     <t>0.02713 (0.23%)</t>
   </si>
   <si>
-    <t>3.057e+21 (26052474104679214612480.00%)</t>
-  </si>
-  <si>
     <t>468.6 (4100.83%)</t>
   </si>
   <si>
@@ -748,9 +721,6 @@
     <t>0.02707 (0.24%)</t>
   </si>
   <si>
-    <t>3.057e+21 (26755350354228328529920.00%)</t>
-  </si>
-  <si>
     <t>Case VII</t>
   </si>
   <si>
@@ -857,6 +827,14 @@
   </si>
   <si>
     <t>-0.01981 (-0.30%)</t>
+  </si>
+  <si>
+    <t>4.106e+68 (nan%)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>3.057e+21 (nan%)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -875,6 +853,8 @@
       <b/>
       <sz val="11"/>
       <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="9"/>
@@ -892,7 +872,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -915,18 +895,65 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1231,25 +1258,35 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K72"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="4" max="4" width="11.1328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.1328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.1328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.19921875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20.6640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C1" s="1"/>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2" t="s">
+      <c r="E1" s="8"/>
+      <c r="F1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2" t="s">
+      <c r="G1" s="8"/>
+      <c r="H1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2" t="s">
+      <c r="I1" s="8"/>
+      <c r="J1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="K1" s="2"/>
+      <c r="K1" s="8"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C2" s="1"/>
@@ -1290,7 +1327,7 @@
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="5" t="s">
         <v>9</v>
       </c>
       <c r="B4" s="1" t="s">
@@ -1299,25 +1336,25 @@
       <c r="C4" s="1">
         <v>1</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="2">
         <v>0.405229999916628</v>
       </c>
       <c r="E4" t="s">
         <v>11</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="2">
         <v>0.42856599995866418</v>
       </c>
       <c r="G4" t="s">
         <v>12</v>
       </c>
-      <c r="H4">
+      <c r="H4" s="2">
         <v>0.62097589997574687</v>
       </c>
       <c r="I4" t="s">
         <v>13</v>
       </c>
-      <c r="J4">
+      <c r="J4" s="2">
         <v>0.6758925000904128</v>
       </c>
       <c r="K4" t="s">
@@ -1325,32 +1362,32 @@
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A5" s="2"/>
+      <c r="A5" s="6"/>
       <c r="B5" s="1" t="s">
         <v>15</v>
       </c>
       <c r="C5" s="1">
         <v>1</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="2">
         <v>2.8924740999937062</v>
       </c>
       <c r="E5" t="s">
         <v>16</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="2">
         <v>3.8481023000786081</v>
       </c>
       <c r="G5" t="s">
         <v>17</v>
       </c>
-      <c r="H5">
+      <c r="H5" s="2">
         <v>5.5486123999580741</v>
       </c>
       <c r="I5" t="s">
         <v>18</v>
       </c>
-      <c r="J5">
+      <c r="J5" s="2">
         <v>6.6601789999986067</v>
       </c>
       <c r="K5" t="s">
@@ -1358,32 +1395,32 @@
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A6" s="2"/>
+      <c r="A6" s="7"/>
       <c r="B6" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C6" s="1">
         <v>1</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="2">
         <v>29.0658381000394</v>
       </c>
       <c r="E6" t="s">
         <v>21</v>
       </c>
-      <c r="F6">
+      <c r="F6" s="2">
         <v>40.384402700001367</v>
       </c>
       <c r="G6" t="s">
         <v>22</v>
       </c>
-      <c r="H6">
+      <c r="H6" s="2">
         <v>88.86462709994521</v>
       </c>
       <c r="I6" t="s">
         <v>23</v>
       </c>
-      <c r="J6">
+      <c r="J6" s="2">
         <v>101.9920106999343</v>
       </c>
       <c r="K6" t="s">
@@ -1391,34 +1428,34 @@
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="5" t="s">
         <v>10</v>
       </c>
       <c r="C7" s="1">
         <v>95</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="3">
         <v>0.2677657000022009</v>
       </c>
       <c r="E7" t="s">
         <v>26</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="3">
         <v>0.24551729997619989</v>
       </c>
       <c r="G7" t="s">
         <v>27</v>
       </c>
-      <c r="H7">
+      <c r="H7" s="3">
         <v>0.46548949996940792</v>
       </c>
       <c r="I7" t="s">
         <v>28</v>
       </c>
-      <c r="J7">
+      <c r="J7" s="3">
         <v>0.39034099993295968</v>
       </c>
       <c r="K7" t="s">
@@ -1426,70 +1463,78 @@
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
+      <c r="A8" s="6"/>
+      <c r="B8" s="6"/>
       <c r="C8" s="1">
         <v>100</v>
       </c>
+      <c r="D8" s="4"/>
       <c r="E8" t="s">
         <v>30</v>
       </c>
+      <c r="F8" s="4"/>
       <c r="G8" t="s">
         <v>31</v>
       </c>
+      <c r="H8" s="4"/>
       <c r="I8" t="s">
         <v>32</v>
       </c>
+      <c r="J8" s="4"/>
       <c r="K8" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
+      <c r="A9" s="6"/>
+      <c r="B9" s="7"/>
       <c r="C9" s="1">
         <v>105</v>
       </c>
+      <c r="D9" s="4"/>
       <c r="E9" t="s">
         <v>34</v>
       </c>
+      <c r="F9" s="4"/>
       <c r="G9" t="s">
         <v>35</v>
       </c>
+      <c r="H9" s="4"/>
       <c r="I9" t="s">
         <v>36</v>
       </c>
+      <c r="J9" s="4"/>
       <c r="K9" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2" t="s">
+      <c r="A10" s="6"/>
+      <c r="B10" s="5" t="s">
         <v>15</v>
       </c>
       <c r="C10" s="1">
         <v>95</v>
       </c>
-      <c r="D10">
+      <c r="D10" s="3">
         <v>1.5047430000267921</v>
       </c>
       <c r="E10" t="s">
         <v>38</v>
       </c>
-      <c r="F10">
+      <c r="F10" s="3">
         <v>1.963980600005016</v>
       </c>
       <c r="G10" t="s">
         <v>39</v>
       </c>
-      <c r="H10">
+      <c r="H10" s="3">
         <v>2.9798647999996319</v>
       </c>
       <c r="I10" t="s">
         <v>40</v>
       </c>
-      <c r="J10">
+      <c r="J10" s="3">
         <v>3.39737579994835</v>
       </c>
       <c r="K10" t="s">
@@ -1497,70 +1542,78 @@
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
+      <c r="A11" s="6"/>
+      <c r="B11" s="6"/>
       <c r="C11" s="1">
         <v>100</v>
       </c>
+      <c r="D11" s="4"/>
       <c r="E11" t="s">
         <v>42</v>
       </c>
+      <c r="F11" s="4"/>
       <c r="G11" t="s">
         <v>43</v>
       </c>
+      <c r="H11" s="4"/>
       <c r="I11" t="s">
         <v>44</v>
       </c>
+      <c r="J11" s="4"/>
       <c r="K11" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
+      <c r="A12" s="6"/>
+      <c r="B12" s="7"/>
       <c r="C12" s="1">
         <v>105</v>
       </c>
+      <c r="D12" s="4"/>
       <c r="E12" t="s">
         <v>46</v>
       </c>
+      <c r="F12" s="4"/>
       <c r="G12" t="s">
         <v>47</v>
       </c>
+      <c r="H12" s="4"/>
       <c r="I12" t="s">
         <v>48</v>
       </c>
+      <c r="J12" s="4"/>
       <c r="K12" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2" t="s">
+      <c r="A13" s="6"/>
+      <c r="B13" s="5" t="s">
         <v>20</v>
       </c>
       <c r="C13" s="1">
         <v>95</v>
       </c>
-      <c r="D13">
+      <c r="D13" s="3">
         <v>14.52534100005869</v>
       </c>
       <c r="E13" t="s">
         <v>50</v>
       </c>
-      <c r="F13">
+      <c r="F13" s="3">
         <v>20.233092900016349</v>
       </c>
       <c r="G13" t="s">
         <v>51</v>
       </c>
-      <c r="H13">
+      <c r="H13" s="3">
         <v>29.562941399984989</v>
       </c>
       <c r="I13" t="s">
         <v>52</v>
       </c>
-      <c r="J13">
+      <c r="J13" s="3">
         <v>48.585087500046939</v>
       </c>
       <c r="K13" t="s">
@@ -1568,72 +1621,80 @@
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
+      <c r="A14" s="6"/>
+      <c r="B14" s="6"/>
       <c r="C14" s="1">
         <v>100</v>
       </c>
+      <c r="D14" s="4"/>
       <c r="E14" t="s">
         <v>54</v>
       </c>
+      <c r="F14" s="4"/>
       <c r="G14" t="s">
         <v>55</v>
       </c>
+      <c r="H14" s="4"/>
       <c r="I14" t="s">
         <v>56</v>
       </c>
+      <c r="J14" s="4"/>
       <c r="K14" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
+      <c r="A15" s="7"/>
+      <c r="B15" s="7"/>
       <c r="C15" s="1">
         <v>105</v>
       </c>
+      <c r="D15" s="4"/>
       <c r="E15" t="s">
         <v>58</v>
       </c>
+      <c r="F15" s="4"/>
       <c r="G15" t="s">
         <v>59</v>
       </c>
+      <c r="H15" s="4"/>
       <c r="I15" t="s">
         <v>60</v>
       </c>
+      <c r="J15" s="4"/>
       <c r="K15" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="5" t="s">
         <v>10</v>
       </c>
       <c r="C16" s="1">
         <v>95</v>
       </c>
-      <c r="D16">
+      <c r="D16" s="3">
         <v>0.238945999997668</v>
       </c>
       <c r="E16" t="s">
         <v>63</v>
       </c>
-      <c r="F16">
+      <c r="F16" s="3">
         <v>0.24176189990248531</v>
       </c>
       <c r="G16" t="s">
         <v>64</v>
       </c>
-      <c r="H16">
+      <c r="H16" s="3">
         <v>0.3870247999439016</v>
       </c>
       <c r="I16" t="s">
         <v>65</v>
       </c>
-      <c r="J16">
+      <c r="J16" s="3">
         <v>0.44235779996961361</v>
       </c>
       <c r="K16" t="s">
@@ -1641,70 +1702,78 @@
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
+      <c r="A17" s="6"/>
+      <c r="B17" s="6"/>
       <c r="C17" s="1">
         <v>100</v>
       </c>
+      <c r="D17" s="4"/>
       <c r="E17" t="s">
         <v>67</v>
       </c>
+      <c r="F17" s="4"/>
       <c r="G17" t="s">
         <v>68</v>
       </c>
+      <c r="H17" s="4"/>
       <c r="I17" t="s">
         <v>69</v>
       </c>
+      <c r="J17" s="4"/>
       <c r="K17" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A18" s="2"/>
-      <c r="B18" s="2"/>
+      <c r="A18" s="6"/>
+      <c r="B18" s="7"/>
       <c r="C18" s="1">
         <v>105</v>
       </c>
+      <c r="D18" s="4"/>
       <c r="E18" t="s">
         <v>71</v>
       </c>
+      <c r="F18" s="4"/>
       <c r="G18" t="s">
         <v>72</v>
       </c>
+      <c r="H18" s="4"/>
       <c r="I18" t="s">
         <v>73</v>
       </c>
+      <c r="J18" s="4"/>
       <c r="K18" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A19" s="2"/>
-      <c r="B19" s="2" t="s">
+      <c r="A19" s="6"/>
+      <c r="B19" s="5" t="s">
         <v>15</v>
       </c>
       <c r="C19" s="1">
         <v>95</v>
       </c>
-      <c r="D19">
+      <c r="D19" s="3">
         <v>1.4755197999766101</v>
       </c>
       <c r="E19" t="s">
         <v>75</v>
       </c>
-      <c r="F19">
+      <c r="F19" s="3">
         <v>1.9966578999301421</v>
       </c>
       <c r="G19" t="s">
         <v>76</v>
       </c>
-      <c r="H19">
+      <c r="H19" s="3">
         <v>2.863436799962074</v>
       </c>
       <c r="I19" t="s">
         <v>77</v>
       </c>
-      <c r="J19">
+      <c r="J19" s="3">
         <v>3.373646300053224</v>
       </c>
       <c r="K19" t="s">
@@ -1712,70 +1781,78 @@
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A20" s="2"/>
-      <c r="B20" s="2"/>
+      <c r="A20" s="6"/>
+      <c r="B20" s="6"/>
       <c r="C20" s="1">
         <v>100</v>
       </c>
+      <c r="D20" s="4"/>
       <c r="E20" t="s">
         <v>79</v>
       </c>
+      <c r="F20" s="4"/>
       <c r="G20" t="s">
         <v>80</v>
       </c>
+      <c r="H20" s="4"/>
       <c r="I20" t="s">
         <v>81</v>
       </c>
+      <c r="J20" s="4"/>
       <c r="K20" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A21" s="2"/>
-      <c r="B21" s="2"/>
+      <c r="A21" s="6"/>
+      <c r="B21" s="7"/>
       <c r="C21" s="1">
         <v>105</v>
       </c>
+      <c r="D21" s="4"/>
       <c r="E21" t="s">
         <v>83</v>
       </c>
+      <c r="F21" s="4"/>
       <c r="G21" t="s">
         <v>84</v>
       </c>
+      <c r="H21" s="4"/>
       <c r="I21" t="s">
         <v>85</v>
       </c>
+      <c r="J21" s="4"/>
       <c r="K21" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A22" s="2"/>
-      <c r="B22" s="2" t="s">
+      <c r="A22" s="6"/>
+      <c r="B22" s="5" t="s">
         <v>20</v>
       </c>
       <c r="C22" s="1">
         <v>95</v>
       </c>
-      <c r="D22">
+      <c r="D22" s="3">
         <v>14.46036919998005</v>
       </c>
       <c r="E22" t="s">
         <v>87</v>
       </c>
-      <c r="F22">
+      <c r="F22" s="3">
         <v>19.967838000040501</v>
       </c>
       <c r="G22" t="s">
         <v>88</v>
       </c>
-      <c r="H22">
+      <c r="H22" s="3">
         <v>28.54840089997742</v>
       </c>
       <c r="I22" t="s">
         <v>89</v>
       </c>
-      <c r="J22">
+      <c r="J22" s="3">
         <v>48.517248400021337</v>
       </c>
       <c r="K22" t="s">
@@ -1783,72 +1860,80 @@
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A23" s="2"/>
-      <c r="B23" s="2"/>
+      <c r="A23" s="6"/>
+      <c r="B23" s="6"/>
       <c r="C23" s="1">
         <v>100</v>
       </c>
+      <c r="D23" s="4"/>
       <c r="E23" t="s">
         <v>90</v>
       </c>
+      <c r="F23" s="4"/>
       <c r="G23" t="s">
         <v>91</v>
       </c>
+      <c r="H23" s="4"/>
       <c r="I23" t="s">
         <v>92</v>
       </c>
+      <c r="J23" s="4"/>
       <c r="K23" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A24" s="2"/>
-      <c r="B24" s="2"/>
+      <c r="A24" s="7"/>
+      <c r="B24" s="7"/>
       <c r="C24" s="1">
         <v>105</v>
       </c>
+      <c r="D24" s="4"/>
       <c r="E24" t="s">
         <v>94</v>
       </c>
+      <c r="F24" s="4"/>
       <c r="G24" t="s">
         <v>95</v>
       </c>
+      <c r="H24" s="4"/>
       <c r="I24" t="s">
         <v>96</v>
       </c>
+      <c r="J24" s="4"/>
       <c r="K24" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A25" s="2" t="s">
+      <c r="A25" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="B25" s="5" t="s">
         <v>10</v>
       </c>
       <c r="C25" s="1">
         <v>47</v>
       </c>
-      <c r="D25">
+      <c r="D25" s="3">
         <v>8.9171500061638653E-2</v>
       </c>
       <c r="E25" t="s">
         <v>99</v>
       </c>
-      <c r="F25">
+      <c r="F25" s="3">
         <v>8.3611599984578788E-2</v>
       </c>
       <c r="G25" t="s">
         <v>100</v>
       </c>
-      <c r="H25">
+      <c r="H25" s="3">
         <v>0.10615459992550309</v>
       </c>
       <c r="I25" t="s">
         <v>101</v>
       </c>
-      <c r="J25">
+      <c r="J25" s="3">
         <v>0.14980510005261749</v>
       </c>
       <c r="K25" t="s">
@@ -1856,108 +1941,124 @@
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A26" s="2"/>
-      <c r="B26" s="2"/>
+      <c r="A26" s="6"/>
+      <c r="B26" s="6"/>
       <c r="C26" s="1">
         <v>48</v>
       </c>
+      <c r="D26" s="4"/>
       <c r="E26" t="s">
         <v>103</v>
       </c>
+      <c r="F26" s="4"/>
       <c r="G26" t="s">
         <v>104</v>
       </c>
+      <c r="H26" s="4"/>
       <c r="I26" t="s">
         <v>105</v>
       </c>
+      <c r="J26" s="4"/>
       <c r="K26" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A27" s="2"/>
-      <c r="B27" s="2"/>
+      <c r="A27" s="6"/>
+      <c r="B27" s="6"/>
       <c r="C27" s="1">
         <v>49</v>
       </c>
+      <c r="D27" s="4"/>
       <c r="E27" t="s">
         <v>107</v>
       </c>
+      <c r="F27" s="4"/>
       <c r="G27" t="s">
         <v>108</v>
       </c>
+      <c r="H27" s="4"/>
       <c r="I27" t="s">
         <v>109</v>
       </c>
+      <c r="J27" s="4"/>
       <c r="K27" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A28" s="2"/>
-      <c r="B28" s="2"/>
+      <c r="A28" s="6"/>
+      <c r="B28" s="6"/>
       <c r="C28" s="1">
         <v>50</v>
       </c>
+      <c r="D28" s="4"/>
       <c r="E28" t="s">
         <v>111</v>
       </c>
+      <c r="F28" s="4"/>
       <c r="G28" t="s">
         <v>112</v>
       </c>
+      <c r="H28" s="4"/>
       <c r="I28" t="s">
         <v>113</v>
       </c>
+      <c r="J28" s="4"/>
       <c r="K28" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A29" s="2"/>
-      <c r="B29" s="2"/>
+      <c r="A29" s="6"/>
+      <c r="B29" s="7"/>
       <c r="C29" s="1">
         <v>51</v>
       </c>
+      <c r="D29" s="4"/>
       <c r="E29" t="s">
         <v>115</v>
       </c>
+      <c r="F29" s="4"/>
       <c r="G29" t="s">
         <v>116</v>
       </c>
+      <c r="H29" s="4"/>
       <c r="I29" t="s">
         <v>117</v>
       </c>
+      <c r="J29" s="4"/>
       <c r="K29" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A30" s="2"/>
-      <c r="B30" s="2" t="s">
+      <c r="A30" s="6"/>
+      <c r="B30" s="5" t="s">
         <v>15</v>
       </c>
       <c r="C30" s="1">
         <v>47</v>
       </c>
-      <c r="D30">
+      <c r="D30" s="3">
         <v>0.32301799999549979</v>
       </c>
       <c r="E30" t="s">
         <v>119</v>
       </c>
-      <c r="F30">
+      <c r="F30" s="3">
         <v>0.43606109998654569</v>
       </c>
       <c r="G30" t="s">
         <v>120</v>
       </c>
-      <c r="H30">
+      <c r="H30" s="3">
         <v>0.60521419998258352</v>
       </c>
       <c r="I30" t="s">
         <v>121</v>
       </c>
-      <c r="J30">
+      <c r="J30" s="3">
         <v>0.70288489991798997</v>
       </c>
       <c r="K30" t="s">
@@ -1965,108 +2066,124 @@
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A31" s="2"/>
-      <c r="B31" s="2"/>
+      <c r="A31" s="6"/>
+      <c r="B31" s="6"/>
       <c r="C31" s="1">
         <v>48</v>
       </c>
+      <c r="D31" s="4"/>
       <c r="E31" t="s">
         <v>123</v>
       </c>
+      <c r="F31" s="4"/>
       <c r="G31" t="s">
         <v>124</v>
       </c>
+      <c r="H31" s="4"/>
       <c r="I31" t="s">
         <v>125</v>
       </c>
+      <c r="J31" s="4"/>
       <c r="K31" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A32" s="2"/>
-      <c r="B32" s="2"/>
+      <c r="A32" s="6"/>
+      <c r="B32" s="6"/>
       <c r="C32" s="1">
         <v>49</v>
       </c>
+      <c r="D32" s="4"/>
       <c r="E32" t="s">
         <v>127</v>
       </c>
+      <c r="F32" s="4"/>
       <c r="G32" t="s">
         <v>128</v>
       </c>
+      <c r="H32" s="4"/>
       <c r="I32" t="s">
         <v>129</v>
       </c>
+      <c r="J32" s="4"/>
       <c r="K32" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A33" s="2"/>
-      <c r="B33" s="2"/>
+      <c r="A33" s="6"/>
+      <c r="B33" s="6"/>
       <c r="C33" s="1">
         <v>50</v>
       </c>
+      <c r="D33" s="4"/>
       <c r="E33" t="s">
         <v>131</v>
       </c>
+      <c r="F33" s="4"/>
       <c r="G33" t="s">
         <v>132</v>
       </c>
+      <c r="H33" s="4"/>
       <c r="I33" t="s">
         <v>133</v>
       </c>
+      <c r="J33" s="4"/>
       <c r="K33" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A34" s="2"/>
-      <c r="B34" s="2"/>
+      <c r="A34" s="6"/>
+      <c r="B34" s="7"/>
       <c r="C34" s="1">
         <v>51</v>
       </c>
+      <c r="D34" s="4"/>
       <c r="E34" t="s">
         <v>135</v>
       </c>
+      <c r="F34" s="4"/>
       <c r="G34" t="s">
         <v>136</v>
       </c>
+      <c r="H34" s="4"/>
       <c r="I34" t="s">
         <v>137</v>
       </c>
+      <c r="J34" s="4"/>
       <c r="K34" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A35" s="2"/>
-      <c r="B35" s="2" t="s">
+      <c r="A35" s="6"/>
+      <c r="B35" s="5" t="s">
         <v>20</v>
       </c>
       <c r="C35" s="1">
         <v>47</v>
       </c>
-      <c r="D35">
+      <c r="D35" s="3">
         <v>3.001315100002103</v>
       </c>
       <c r="E35" t="s">
         <v>139</v>
       </c>
-      <c r="F35">
+      <c r="F35" s="3">
         <v>4.0081003999803224</v>
       </c>
       <c r="G35" t="s">
         <v>140</v>
       </c>
-      <c r="H35">
+      <c r="H35" s="3">
         <v>5.7636176000814876</v>
       </c>
       <c r="I35" t="s">
         <v>141</v>
       </c>
-      <c r="J35">
+      <c r="J35" s="3">
         <v>10.02923349989578</v>
       </c>
       <c r="K35" t="s">
@@ -2074,110 +2191,126 @@
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A36" s="2"/>
-      <c r="B36" s="2"/>
+      <c r="A36" s="6"/>
+      <c r="B36" s="6"/>
       <c r="C36" s="1">
         <v>48</v>
       </c>
+      <c r="D36" s="4"/>
       <c r="E36" t="s">
         <v>143</v>
       </c>
+      <c r="F36" s="4"/>
       <c r="G36" t="s">
         <v>144</v>
       </c>
+      <c r="H36" s="4"/>
       <c r="I36" t="s">
         <v>145</v>
       </c>
+      <c r="J36" s="4"/>
       <c r="K36" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A37" s="2"/>
-      <c r="B37" s="2"/>
+      <c r="A37" s="6"/>
+      <c r="B37" s="6"/>
       <c r="C37" s="1">
         <v>49</v>
       </c>
+      <c r="D37" s="4"/>
       <c r="E37" t="s">
         <v>147</v>
       </c>
+      <c r="F37" s="4"/>
       <c r="G37" t="s">
         <v>148</v>
       </c>
+      <c r="H37" s="4"/>
       <c r="I37" t="s">
         <v>149</v>
       </c>
+      <c r="J37" s="4"/>
       <c r="K37" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A38" s="2"/>
-      <c r="B38" s="2"/>
+      <c r="A38" s="6"/>
+      <c r="B38" s="6"/>
       <c r="C38" s="1">
         <v>50</v>
       </c>
+      <c r="D38" s="4"/>
       <c r="E38" t="s">
         <v>151</v>
       </c>
+      <c r="F38" s="4"/>
       <c r="G38" t="s">
         <v>152</v>
       </c>
+      <c r="H38" s="4"/>
       <c r="I38" t="s">
         <v>153</v>
       </c>
+      <c r="J38" s="4"/>
       <c r="K38" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A39" s="2"/>
-      <c r="B39" s="2"/>
+      <c r="A39" s="7"/>
+      <c r="B39" s="7"/>
       <c r="C39" s="1">
         <v>51</v>
       </c>
+      <c r="D39" s="4"/>
       <c r="E39" t="s">
         <v>155</v>
       </c>
+      <c r="F39" s="4"/>
       <c r="G39" t="s">
         <v>156</v>
       </c>
+      <c r="H39" s="4"/>
       <c r="I39" t="s">
         <v>157</v>
       </c>
+      <c r="J39" s="4"/>
       <c r="K39" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A40" s="2" t="s">
+      <c r="A40" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="B40" s="2" t="s">
+      <c r="B40" s="5" t="s">
         <v>10</v>
       </c>
       <c r="C40" s="1">
         <v>10</v>
       </c>
-      <c r="D40">
+      <c r="D40" s="3">
         <v>8.7301699910312891E-2</v>
       </c>
       <c r="E40" t="s">
         <v>160</v>
       </c>
-      <c r="F40">
+      <c r="F40" s="3">
         <v>8.4547300008125603E-2</v>
       </c>
       <c r="G40" t="s">
         <v>161</v>
       </c>
-      <c r="H40">
+      <c r="H40" s="3">
         <v>0.1103219001088291</v>
       </c>
       <c r="I40" t="s">
         <v>162</v>
       </c>
-      <c r="J40">
+      <c r="J40" s="3">
         <v>0.12990299996454269</v>
       </c>
       <c r="K40" t="s">
@@ -2185,70 +2318,78 @@
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A41" s="2"/>
-      <c r="B41" s="2"/>
+      <c r="A41" s="6"/>
+      <c r="B41" s="6"/>
       <c r="C41" s="1">
         <v>20</v>
       </c>
+      <c r="D41" s="4"/>
       <c r="E41" t="s">
         <v>164</v>
       </c>
+      <c r="F41" s="4"/>
       <c r="G41" t="s">
         <v>165</v>
       </c>
+      <c r="H41" s="4"/>
       <c r="I41" t="s">
         <v>166</v>
       </c>
+      <c r="J41" s="4"/>
       <c r="K41" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A42" s="2"/>
-      <c r="B42" s="2"/>
+      <c r="A42" s="6"/>
+      <c r="B42" s="7"/>
       <c r="C42" s="1">
         <v>40</v>
       </c>
+      <c r="D42" s="4"/>
       <c r="E42" t="s">
         <v>168</v>
       </c>
+      <c r="F42" s="4"/>
       <c r="G42" t="s">
         <v>169</v>
       </c>
+      <c r="H42" s="4"/>
       <c r="I42" t="s">
         <v>170</v>
       </c>
+      <c r="J42" s="4"/>
       <c r="K42" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A43" s="2"/>
-      <c r="B43" s="2" t="s">
+      <c r="A43" s="6"/>
+      <c r="B43" s="5" t="s">
         <v>15</v>
       </c>
       <c r="C43" s="1">
         <v>10</v>
       </c>
-      <c r="D43">
+      <c r="D43" s="3">
         <v>0.329887600033544</v>
       </c>
       <c r="E43" t="s">
         <v>172</v>
       </c>
-      <c r="F43">
+      <c r="F43" s="3">
         <v>0.42904950003139669</v>
       </c>
       <c r="G43" t="s">
         <v>173</v>
       </c>
-      <c r="H43">
+      <c r="H43" s="3">
         <v>0.58943910000380129</v>
       </c>
       <c r="I43" t="s">
         <v>174</v>
       </c>
-      <c r="J43">
+      <c r="J43" s="3">
         <v>0.70071749994531274</v>
       </c>
       <c r="K43" t="s">
@@ -2256,70 +2397,78 @@
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A44" s="2"/>
-      <c r="B44" s="2"/>
+      <c r="A44" s="6"/>
+      <c r="B44" s="6"/>
       <c r="C44" s="1">
         <v>20</v>
       </c>
+      <c r="D44" s="4"/>
       <c r="E44" t="s">
         <v>176</v>
       </c>
+      <c r="F44" s="4"/>
       <c r="G44" t="s">
         <v>177</v>
       </c>
+      <c r="H44" s="4"/>
       <c r="I44" t="s">
         <v>178</v>
       </c>
+      <c r="J44" s="4"/>
       <c r="K44" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A45" s="2"/>
-      <c r="B45" s="2"/>
+      <c r="A45" s="6"/>
+      <c r="B45" s="7"/>
       <c r="C45" s="1">
         <v>40</v>
       </c>
+      <c r="D45" s="4"/>
       <c r="E45" t="s">
         <v>180</v>
       </c>
+      <c r="F45" s="4"/>
       <c r="G45" t="s">
         <v>181</v>
       </c>
+      <c r="H45" s="4"/>
       <c r="I45" t="s">
         <v>182</v>
       </c>
+      <c r="J45" s="4"/>
       <c r="K45" t="s">
         <v>183</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A46" s="2"/>
-      <c r="B46" s="2" t="s">
+      <c r="A46" s="6"/>
+      <c r="B46" s="5" t="s">
         <v>20</v>
       </c>
       <c r="C46" s="1">
         <v>10</v>
       </c>
-      <c r="D46">
+      <c r="D46" s="3">
         <v>2.9262787998886779</v>
       </c>
       <c r="E46" t="s">
         <v>184</v>
       </c>
-      <c r="F46">
+      <c r="F46" s="3">
         <v>4.0733267000177884</v>
       </c>
       <c r="G46" t="s">
         <v>185</v>
       </c>
-      <c r="H46">
+      <c r="H46" s="3">
         <v>5.720168299973011</v>
       </c>
       <c r="I46" t="s">
         <v>186</v>
       </c>
-      <c r="J46">
+      <c r="J46" s="3">
         <v>9.9833600999554619</v>
       </c>
       <c r="K46" t="s">
@@ -2327,72 +2476,80 @@
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A47" s="2"/>
-      <c r="B47" s="2"/>
+      <c r="A47" s="6"/>
+      <c r="B47" s="6"/>
       <c r="C47" s="1">
         <v>20</v>
       </c>
+      <c r="D47" s="4"/>
       <c r="E47" t="s">
         <v>188</v>
       </c>
+      <c r="F47" s="4"/>
       <c r="G47" t="s">
         <v>189</v>
       </c>
+      <c r="H47" s="4"/>
       <c r="I47" t="s">
         <v>190</v>
       </c>
+      <c r="J47" s="4"/>
       <c r="K47" t="s">
         <v>191</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A48" s="2"/>
-      <c r="B48" s="2"/>
+      <c r="A48" s="7"/>
+      <c r="B48" s="7"/>
       <c r="C48" s="1">
         <v>40</v>
       </c>
+      <c r="D48" s="4"/>
       <c r="E48" t="s">
         <v>192</v>
       </c>
+      <c r="F48" s="4"/>
       <c r="G48" t="s">
         <v>193</v>
       </c>
+      <c r="H48" s="4"/>
       <c r="I48" t="s">
         <v>194</v>
       </c>
+      <c r="J48" s="4"/>
       <c r="K48" t="s">
         <v>195</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A49" s="2" t="s">
+      <c r="A49" s="5" t="s">
         <v>196</v>
       </c>
-      <c r="B49" s="2" t="s">
+      <c r="B49" s="5" t="s">
         <v>10</v>
       </c>
       <c r="C49" s="1">
         <v>47</v>
       </c>
-      <c r="D49">
+      <c r="D49" s="3">
         <v>0.38312290003523231</v>
       </c>
       <c r="E49" t="s">
         <v>197</v>
       </c>
-      <c r="F49">
+      <c r="F49" s="3">
         <v>0.43022370000835508</v>
       </c>
       <c r="G49" t="s">
         <v>198</v>
       </c>
-      <c r="H49">
+      <c r="H49" s="3">
         <v>0.78730580001138151</v>
       </c>
       <c r="I49" t="s">
         <v>199</v>
       </c>
-      <c r="J49">
+      <c r="J49" s="3">
         <v>0.70451229996979237</v>
       </c>
       <c r="K49" t="s">
@@ -2400,545 +2557,689 @@
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A50" s="2"/>
-      <c r="B50" s="2"/>
+      <c r="A50" s="6"/>
+      <c r="B50" s="6"/>
       <c r="C50" s="1">
         <v>48</v>
       </c>
+      <c r="D50" s="4"/>
       <c r="E50" t="s">
         <v>197</v>
       </c>
+      <c r="F50" s="4"/>
       <c r="G50" t="s">
         <v>200</v>
       </c>
+      <c r="H50" s="4"/>
       <c r="I50" t="s">
         <v>201</v>
       </c>
+      <c r="J50" s="4"/>
       <c r="K50" t="s">
         <v>197</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A51" s="2"/>
-      <c r="B51" s="2"/>
+      <c r="A51" s="6"/>
+      <c r="B51" s="6"/>
       <c r="C51" s="1">
         <v>49</v>
       </c>
+      <c r="D51" s="4"/>
       <c r="E51" t="s">
         <v>197</v>
       </c>
+      <c r="F51" s="4"/>
       <c r="G51" t="s">
         <v>202</v>
       </c>
+      <c r="H51" s="4"/>
       <c r="I51" t="s">
         <v>203</v>
       </c>
+      <c r="J51" s="4"/>
       <c r="K51" t="s">
         <v>197</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A52" s="2"/>
-      <c r="B52" s="2"/>
+      <c r="A52" s="6"/>
+      <c r="B52" s="6"/>
       <c r="C52" s="1">
         <v>50</v>
       </c>
+      <c r="D52" s="4"/>
       <c r="E52" t="s">
         <v>197</v>
       </c>
+      <c r="F52" s="4"/>
       <c r="G52" t="s">
         <v>204</v>
       </c>
+      <c r="H52" s="4"/>
       <c r="I52" t="s">
         <v>205</v>
       </c>
+      <c r="J52" s="4"/>
       <c r="K52" t="s">
         <v>197</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A53" s="2"/>
-      <c r="B53" s="2"/>
+      <c r="A53" s="6"/>
+      <c r="B53" s="7"/>
       <c r="C53" s="1">
         <v>51</v>
       </c>
+      <c r="D53" s="4"/>
       <c r="E53" t="s">
         <v>197</v>
       </c>
+      <c r="F53" s="4"/>
       <c r="G53" t="s">
         <v>206</v>
       </c>
+      <c r="H53" s="4"/>
       <c r="I53" t="s">
         <v>207</v>
       </c>
+      <c r="J53" s="4"/>
       <c r="K53" t="s">
         <v>197</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A54" s="2"/>
-      <c r="B54" s="2" t="s">
+      <c r="A54" s="6"/>
+      <c r="B54" s="5" t="s">
         <v>15</v>
       </c>
       <c r="C54" s="1">
         <v>47</v>
       </c>
-      <c r="D54">
+      <c r="D54" s="3">
         <v>2.8947976999916141</v>
       </c>
       <c r="E54" t="s">
         <v>197</v>
       </c>
-      <c r="F54">
+      <c r="F54" s="3">
         <v>3.8898246999597181</v>
       </c>
       <c r="G54" t="s">
         <v>208</v>
       </c>
-      <c r="H54">
+      <c r="H54" s="3">
         <v>5.8676512000383809</v>
       </c>
       <c r="I54" t="s">
         <v>209</v>
       </c>
-      <c r="J54">
+      <c r="J54" s="3">
         <v>6.6754493000917137</v>
       </c>
       <c r="K54" t="s">
-        <v>210</v>
+        <v>269</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A55" s="2"/>
-      <c r="B55" s="2"/>
+      <c r="A55" s="6"/>
+      <c r="B55" s="6"/>
       <c r="C55" s="1">
         <v>48</v>
       </c>
+      <c r="D55" s="4"/>
       <c r="E55" t="s">
         <v>197</v>
       </c>
+      <c r="F55" s="4"/>
       <c r="G55" t="s">
+        <v>210</v>
+      </c>
+      <c r="H55" s="4"/>
+      <c r="I55" t="s">
         <v>211</v>
       </c>
-      <c r="I55" t="s">
-        <v>212</v>
-      </c>
+      <c r="J55" s="4"/>
       <c r="K55" t="s">
-        <v>213</v>
+        <v>269</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A56" s="2"/>
-      <c r="B56" s="2"/>
+      <c r="A56" s="6"/>
+      <c r="B56" s="6"/>
       <c r="C56" s="1">
         <v>49</v>
       </c>
+      <c r="D56" s="4"/>
       <c r="E56" t="s">
         <v>197</v>
       </c>
+      <c r="F56" s="4"/>
       <c r="G56" t="s">
-        <v>214</v>
-      </c>
+        <v>212</v>
+      </c>
+      <c r="H56" s="4"/>
       <c r="I56" t="s">
-        <v>215</v>
-      </c>
+        <v>213</v>
+      </c>
+      <c r="J56" s="4"/>
       <c r="K56" t="s">
-        <v>216</v>
+        <v>269</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A57" s="2"/>
-      <c r="B57" s="2"/>
+      <c r="A57" s="6"/>
+      <c r="B57" s="6"/>
       <c r="C57" s="1">
         <v>50</v>
       </c>
+      <c r="D57" s="4"/>
       <c r="E57" t="s">
         <v>197</v>
       </c>
+      <c r="F57" s="4"/>
       <c r="G57" t="s">
-        <v>217</v>
-      </c>
+        <v>214</v>
+      </c>
+      <c r="H57" s="4"/>
       <c r="I57" t="s">
-        <v>218</v>
-      </c>
+        <v>215</v>
+      </c>
+      <c r="J57" s="4"/>
       <c r="K57" t="s">
-        <v>219</v>
+        <v>269</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A58" s="2"/>
-      <c r="B58" s="2"/>
+      <c r="A58" s="6"/>
+      <c r="B58" s="7"/>
       <c r="C58" s="1">
         <v>51</v>
       </c>
+      <c r="D58" s="4"/>
       <c r="E58" t="s">
         <v>197</v>
       </c>
+      <c r="F58" s="4"/>
       <c r="G58" t="s">
-        <v>220</v>
-      </c>
+        <v>216</v>
+      </c>
+      <c r="H58" s="4"/>
       <c r="I58" t="s">
-        <v>221</v>
-      </c>
+        <v>217</v>
+      </c>
+      <c r="J58" s="4"/>
       <c r="K58" t="s">
-        <v>222</v>
+        <v>269</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A59" s="2"/>
-      <c r="B59" s="2" t="s">
+      <c r="A59" s="6"/>
+      <c r="B59" s="5" t="s">
         <v>20</v>
       </c>
       <c r="C59" s="1">
         <v>47</v>
       </c>
-      <c r="D59">
+      <c r="D59" s="3">
         <v>29.223953899927441</v>
       </c>
       <c r="E59" t="s">
-        <v>223</v>
-      </c>
-      <c r="F59">
+        <v>218</v>
+      </c>
+      <c r="F59" s="3">
         <v>55.427861100062728</v>
       </c>
       <c r="G59" t="s">
-        <v>224</v>
-      </c>
-      <c r="H59">
+        <v>219</v>
+      </c>
+      <c r="H59" s="3">
         <v>57.770199500024319</v>
       </c>
       <c r="I59" t="s">
-        <v>225</v>
-      </c>
-      <c r="J59">
+        <v>220</v>
+      </c>
+      <c r="J59" s="3">
         <v>99.37938940001186</v>
       </c>
       <c r="K59" t="s">
-        <v>226</v>
+        <v>270</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A60" s="2"/>
-      <c r="B60" s="2"/>
+      <c r="A60" s="6"/>
+      <c r="B60" s="6"/>
       <c r="C60" s="1">
         <v>48</v>
       </c>
+      <c r="D60" s="4"/>
       <c r="E60" t="s">
-        <v>227</v>
-      </c>
+        <v>221</v>
+      </c>
+      <c r="F60" s="4"/>
       <c r="G60" t="s">
-        <v>228</v>
-      </c>
+        <v>222</v>
+      </c>
+      <c r="H60" s="4"/>
       <c r="I60" t="s">
-        <v>229</v>
-      </c>
+        <v>223</v>
+      </c>
+      <c r="J60" s="4"/>
       <c r="K60" t="s">
-        <v>230</v>
+        <v>270</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A61" s="2"/>
-      <c r="B61" s="2"/>
+      <c r="A61" s="6"/>
+      <c r="B61" s="6"/>
       <c r="C61" s="1">
         <v>49</v>
       </c>
+      <c r="D61" s="4"/>
       <c r="E61" t="s">
-        <v>231</v>
-      </c>
+        <v>224</v>
+      </c>
+      <c r="F61" s="4"/>
       <c r="G61" t="s">
-        <v>232</v>
-      </c>
+        <v>225</v>
+      </c>
+      <c r="H61" s="4"/>
       <c r="I61" t="s">
-        <v>233</v>
-      </c>
+        <v>226</v>
+      </c>
+      <c r="J61" s="4"/>
       <c r="K61" t="s">
-        <v>234</v>
+        <v>270</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A62" s="2"/>
-      <c r="B62" s="2"/>
+      <c r="A62" s="6"/>
+      <c r="B62" s="6"/>
       <c r="C62" s="1">
         <v>50</v>
       </c>
+      <c r="D62" s="4"/>
       <c r="E62" t="s">
-        <v>235</v>
-      </c>
+        <v>227</v>
+      </c>
+      <c r="F62" s="4"/>
       <c r="G62" t="s">
-        <v>236</v>
-      </c>
+        <v>228</v>
+      </c>
+      <c r="H62" s="4"/>
       <c r="I62" t="s">
-        <v>237</v>
-      </c>
+        <v>229</v>
+      </c>
+      <c r="J62" s="4"/>
       <c r="K62" t="s">
-        <v>238</v>
+        <v>270</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A63" s="2"/>
-      <c r="B63" s="2"/>
+      <c r="A63" s="7"/>
+      <c r="B63" s="7"/>
       <c r="C63" s="1">
         <v>51</v>
       </c>
+      <c r="D63" s="4"/>
       <c r="E63" t="s">
-        <v>239</v>
-      </c>
+        <v>230</v>
+      </c>
+      <c r="F63" s="4"/>
       <c r="G63" t="s">
-        <v>240</v>
-      </c>
+        <v>231</v>
+      </c>
+      <c r="H63" s="4"/>
       <c r="I63" t="s">
-        <v>241</v>
-      </c>
+        <v>232</v>
+      </c>
+      <c r="J63" s="4"/>
       <c r="K63" t="s">
-        <v>242</v>
+        <v>270</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A64" s="2" t="s">
-        <v>243</v>
-      </c>
-      <c r="B64" s="2" t="s">
+      <c r="A64" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="B64" s="5" t="s">
         <v>10</v>
       </c>
       <c r="C64" s="1">
         <v>95</v>
       </c>
-      <c r="D64">
+      <c r="D64" s="3">
         <v>0.21036979998461899</v>
       </c>
       <c r="E64" t="s">
-        <v>244</v>
-      </c>
-      <c r="F64">
+        <v>234</v>
+      </c>
+      <c r="F64" s="3">
         <v>0.24970609997399151</v>
       </c>
       <c r="G64" t="s">
-        <v>245</v>
-      </c>
-      <c r="H64">
+        <v>235</v>
+      </c>
+      <c r="H64" s="3">
         <v>0.37662180000916118</v>
       </c>
       <c r="I64" t="s">
-        <v>246</v>
-      </c>
-      <c r="J64">
+        <v>236</v>
+      </c>
+      <c r="J64" s="3">
         <v>0.37422160001005977</v>
       </c>
       <c r="K64" t="s">
-        <v>247</v>
+        <v>237</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A65" s="2"/>
-      <c r="B65" s="2"/>
+      <c r="A65" s="6"/>
+      <c r="B65" s="6"/>
       <c r="C65" s="1">
         <v>100</v>
       </c>
+      <c r="D65" s="4"/>
       <c r="E65" t="s">
-        <v>248</v>
-      </c>
+        <v>238</v>
+      </c>
+      <c r="F65" s="4"/>
       <c r="G65" t="s">
-        <v>249</v>
-      </c>
+        <v>239</v>
+      </c>
+      <c r="H65" s="4"/>
       <c r="I65" t="s">
-        <v>250</v>
-      </c>
+        <v>240</v>
+      </c>
+      <c r="J65" s="4"/>
       <c r="K65" t="s">
-        <v>251</v>
+        <v>241</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A66" s="2"/>
-      <c r="B66" s="2"/>
+      <c r="A66" s="6"/>
+      <c r="B66" s="7"/>
       <c r="C66" s="1">
         <v>105</v>
       </c>
+      <c r="D66" s="4"/>
       <c r="E66" t="s">
-        <v>252</v>
-      </c>
+        <v>242</v>
+      </c>
+      <c r="F66" s="4"/>
       <c r="G66" t="s">
-        <v>253</v>
-      </c>
+        <v>243</v>
+      </c>
+      <c r="H66" s="4"/>
       <c r="I66" t="s">
-        <v>254</v>
-      </c>
+        <v>244</v>
+      </c>
+      <c r="J66" s="4"/>
       <c r="K66" t="s">
-        <v>255</v>
+        <v>245</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A67" s="2"/>
-      <c r="B67" s="2" t="s">
+      <c r="A67" s="6"/>
+      <c r="B67" s="5" t="s">
         <v>15</v>
       </c>
       <c r="C67" s="1">
         <v>95</v>
       </c>
-      <c r="D67">
+      <c r="D67" s="3">
         <v>1.4952732999809091</v>
       </c>
       <c r="E67" t="s">
-        <v>256</v>
-      </c>
-      <c r="F67">
+        <v>246</v>
+      </c>
+      <c r="F67" s="3">
         <v>1.938804800040089</v>
       </c>
       <c r="G67" t="s">
-        <v>257</v>
-      </c>
-      <c r="H67">
+        <v>247</v>
+      </c>
+      <c r="H67" s="3">
         <v>2.9082565000280738</v>
       </c>
       <c r="I67" t="s">
-        <v>258</v>
-      </c>
-      <c r="J67">
+        <v>248</v>
+      </c>
+      <c r="J67" s="3">
         <v>3.3668100000359118</v>
       </c>
       <c r="K67" t="s">
-        <v>259</v>
+        <v>249</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A68" s="2"/>
-      <c r="B68" s="2"/>
+      <c r="A68" s="6"/>
+      <c r="B68" s="6"/>
       <c r="C68" s="1">
         <v>100</v>
       </c>
+      <c r="D68" s="4"/>
       <c r="E68" t="s">
-        <v>260</v>
-      </c>
+        <v>250</v>
+      </c>
+      <c r="F68" s="4"/>
       <c r="G68" t="s">
-        <v>261</v>
-      </c>
+        <v>251</v>
+      </c>
+      <c r="H68" s="4"/>
       <c r="I68" t="s">
-        <v>262</v>
-      </c>
+        <v>252</v>
+      </c>
+      <c r="J68" s="4"/>
       <c r="K68" t="s">
-        <v>263</v>
+        <v>253</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A69" s="2"/>
-      <c r="B69" s="2"/>
+      <c r="A69" s="6"/>
+      <c r="B69" s="7"/>
       <c r="C69" s="1">
         <v>105</v>
       </c>
+      <c r="D69" s="4"/>
       <c r="E69" t="s">
-        <v>264</v>
-      </c>
+        <v>254</v>
+      </c>
+      <c r="F69" s="4"/>
       <c r="G69" t="s">
-        <v>265</v>
-      </c>
+        <v>255</v>
+      </c>
+      <c r="H69" s="4"/>
       <c r="I69" t="s">
-        <v>266</v>
-      </c>
+        <v>256</v>
+      </c>
+      <c r="J69" s="4"/>
       <c r="K69" t="s">
-        <v>267</v>
+        <v>257</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A70" s="2"/>
-      <c r="B70" s="2" t="s">
+      <c r="A70" s="6"/>
+      <c r="B70" s="5" t="s">
         <v>20</v>
       </c>
       <c r="C70" s="1">
         <v>95</v>
       </c>
-      <c r="D70">
+      <c r="D70" s="3">
         <v>14.7206091999542</v>
       </c>
       <c r="E70" t="s">
-        <v>268</v>
-      </c>
-      <c r="F70">
+        <v>258</v>
+      </c>
+      <c r="F70" s="3">
         <v>34.249781799968332</v>
       </c>
       <c r="G70" t="s">
-        <v>269</v>
-      </c>
-      <c r="H70">
+        <v>259</v>
+      </c>
+      <c r="H70" s="3">
         <v>48.121484700008303</v>
       </c>
       <c r="I70" t="s">
-        <v>270</v>
-      </c>
-      <c r="J70">
+        <v>260</v>
+      </c>
+      <c r="J70" s="3">
         <v>52.205460399971336</v>
       </c>
       <c r="K70" t="s">
-        <v>245</v>
+        <v>235</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A71" s="2"/>
-      <c r="B71" s="2"/>
+      <c r="A71" s="6"/>
+      <c r="B71" s="6"/>
       <c r="C71" s="1">
         <v>100</v>
       </c>
+      <c r="D71" s="4"/>
       <c r="E71" t="s">
-        <v>271</v>
-      </c>
+        <v>261</v>
+      </c>
+      <c r="F71" s="4"/>
       <c r="G71" t="s">
-        <v>272</v>
-      </c>
+        <v>262</v>
+      </c>
+      <c r="H71" s="4"/>
       <c r="I71" t="s">
-        <v>273</v>
-      </c>
+        <v>263</v>
+      </c>
+      <c r="J71" s="4"/>
       <c r="K71" t="s">
-        <v>274</v>
+        <v>264</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A72" s="2"/>
-      <c r="B72" s="2"/>
+      <c r="A72" s="7"/>
+      <c r="B72" s="7"/>
       <c r="C72" s="1">
         <v>105</v>
       </c>
+      <c r="D72" s="4"/>
       <c r="E72" t="s">
-        <v>275</v>
-      </c>
+        <v>265</v>
+      </c>
+      <c r="F72" s="4"/>
       <c r="G72" t="s">
-        <v>276</v>
-      </c>
+        <v>266</v>
+      </c>
+      <c r="H72" s="4"/>
       <c r="I72" t="s">
-        <v>277</v>
-      </c>
+        <v>267</v>
+      </c>
+      <c r="J72" s="4"/>
       <c r="K72" t="s">
-        <v>278</v>
+        <v>268</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="29">
+  <mergeCells count="101">
+    <mergeCell ref="B67:B69"/>
+    <mergeCell ref="A49:A63"/>
+    <mergeCell ref="D64:D66"/>
+    <mergeCell ref="J22:J24"/>
+    <mergeCell ref="F64:F66"/>
+    <mergeCell ref="B30:B34"/>
+    <mergeCell ref="A25:A39"/>
+    <mergeCell ref="B64:B66"/>
+    <mergeCell ref="D30:D34"/>
+    <mergeCell ref="F10:F12"/>
+    <mergeCell ref="B54:B58"/>
+    <mergeCell ref="D54:D58"/>
+    <mergeCell ref="H30:H34"/>
+    <mergeCell ref="D40:D42"/>
+    <mergeCell ref="F40:F42"/>
+    <mergeCell ref="J13:J15"/>
+    <mergeCell ref="J64:J66"/>
+    <mergeCell ref="H43:H45"/>
+    <mergeCell ref="A40:A48"/>
+    <mergeCell ref="D49:D53"/>
+    <mergeCell ref="B13:B15"/>
+    <mergeCell ref="D13:D15"/>
+    <mergeCell ref="B19:B21"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="F22:F24"/>
+    <mergeCell ref="H22:H24"/>
+    <mergeCell ref="J35:J39"/>
+    <mergeCell ref="F46:F48"/>
+    <mergeCell ref="J25:J29"/>
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="J7:J9"/>
+    <mergeCell ref="J16:J18"/>
+    <mergeCell ref="J1:K1"/>
+    <mergeCell ref="B49:B53"/>
+    <mergeCell ref="J43:J45"/>
+    <mergeCell ref="A4:A6"/>
+    <mergeCell ref="D19:D21"/>
+    <mergeCell ref="F19:F21"/>
+    <mergeCell ref="B35:B39"/>
+    <mergeCell ref="D35:D39"/>
+    <mergeCell ref="B25:B29"/>
+    <mergeCell ref="B46:B48"/>
+    <mergeCell ref="D46:D48"/>
+    <mergeCell ref="F30:F34"/>
+    <mergeCell ref="J30:J34"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="B40:B42"/>
+    <mergeCell ref="J46:J48"/>
+    <mergeCell ref="H13:H15"/>
+    <mergeCell ref="B16:B18"/>
+    <mergeCell ref="D10:D12"/>
+    <mergeCell ref="B43:B45"/>
+    <mergeCell ref="F7:F9"/>
     <mergeCell ref="A64:A72"/>
-    <mergeCell ref="B46:B48"/>
-    <mergeCell ref="A40:A48"/>
+    <mergeCell ref="H46:H48"/>
     <mergeCell ref="B70:B72"/>
-    <mergeCell ref="B67:B69"/>
-    <mergeCell ref="B64:B66"/>
+    <mergeCell ref="H40:H42"/>
+    <mergeCell ref="D70:D72"/>
+    <mergeCell ref="J40:J42"/>
+    <mergeCell ref="F70:F72"/>
+    <mergeCell ref="B10:B12"/>
+    <mergeCell ref="D7:D9"/>
+    <mergeCell ref="A7:A15"/>
+    <mergeCell ref="D16:D18"/>
+    <mergeCell ref="A16:A24"/>
+    <mergeCell ref="J54:J58"/>
+    <mergeCell ref="J70:J72"/>
+    <mergeCell ref="F13:F15"/>
+    <mergeCell ref="D43:D45"/>
+    <mergeCell ref="H7:H9"/>
+    <mergeCell ref="F43:F45"/>
+    <mergeCell ref="H16:H18"/>
+    <mergeCell ref="H64:H66"/>
+    <mergeCell ref="F59:F63"/>
+    <mergeCell ref="H59:H63"/>
+    <mergeCell ref="J59:J63"/>
+    <mergeCell ref="H70:H72"/>
+    <mergeCell ref="F35:F39"/>
+    <mergeCell ref="H19:H21"/>
+    <mergeCell ref="F49:F53"/>
+    <mergeCell ref="D25:D29"/>
     <mergeCell ref="B7:B9"/>
-    <mergeCell ref="B54:B58"/>
-    <mergeCell ref="B16:B18"/>
+    <mergeCell ref="H67:H69"/>
+    <mergeCell ref="J67:J69"/>
     <mergeCell ref="B59:B63"/>
     <mergeCell ref="B22:B24"/>
-    <mergeCell ref="B35:B39"/>
-    <mergeCell ref="B43:B45"/>
-    <mergeCell ref="B25:B29"/>
-    <mergeCell ref="B10:B12"/>
-    <mergeCell ref="B13:B15"/>
-    <mergeCell ref="B19:B21"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="B40:B42"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="A49:A63"/>
-    <mergeCell ref="B49:B53"/>
-    <mergeCell ref="A4:A6"/>
-    <mergeCell ref="B30:B34"/>
-    <mergeCell ref="A25:A39"/>
-    <mergeCell ref="A7:A15"/>
-    <mergeCell ref="A16:A24"/>
-    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="D59:D63"/>
+    <mergeCell ref="D22:D24"/>
+    <mergeCell ref="H35:H39"/>
+    <mergeCell ref="F25:F29"/>
+    <mergeCell ref="D67:D69"/>
+    <mergeCell ref="F67:F69"/>
+    <mergeCell ref="F54:F58"/>
+    <mergeCell ref="H54:H58"/>
+    <mergeCell ref="F16:F18"/>
+    <mergeCell ref="H10:H12"/>
+    <mergeCell ref="J10:J12"/>
+    <mergeCell ref="J19:J21"/>
+    <mergeCell ref="H49:H53"/>
+    <mergeCell ref="J49:J53"/>
+    <mergeCell ref="H25:H29"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
update figs and tables
</commit_message>
<xml_diff>
--- a/table1_timestep_dts.xlsx
+++ b/table1_timestep_dts.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -943,28 +943,28 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1285,61 +1285,61 @@
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="2"/>
       <c r="B1" s="2"/>
-      <c r="C1" s="8"/>
+      <c r="C1" s="3"/>
       <c r="D1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="10"/>
+      <c r="E1" s="12"/>
       <c r="F1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="10"/>
+      <c r="G1" s="12"/>
       <c r="H1" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="I1" s="10"/>
+      <c r="I1" s="12"/>
       <c r="J1" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="K1" s="10"/>
+      <c r="K1" s="12"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8" t="s">
+      <c r="C2" s="3"/>
+      <c r="D2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="F2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="8" t="s">
+      <c r="G2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="8" t="s">
+      <c r="H2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="I2" s="8" t="s">
+      <c r="I2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="8" t="s">
+      <c r="J2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="K2" s="8" t="s">
+      <c r="K2" s="3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D3" s="2"/>
@@ -1355,10 +1355,10 @@
       <c r="A4" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="8">
+      <c r="C4" s="3">
         <v>1</v>
       </c>
       <c r="D4" s="2">
@@ -1387,11 +1387,11 @@
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A5" s="11"/>
-      <c r="B5" s="8" t="s">
+      <c r="A5" s="10"/>
+      <c r="B5" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="8">
+      <c r="C5" s="3">
         <v>1</v>
       </c>
       <c r="D5" s="2">
@@ -1420,11 +1420,11 @@
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A6" s="12"/>
-      <c r="B6" s="8" t="s">
+      <c r="A6" s="11"/>
+      <c r="B6" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="8">
+      <c r="C6" s="3">
         <v>1</v>
       </c>
       <c r="D6" s="2">
@@ -1459,28 +1459,28 @@
       <c r="B7" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="8">
+      <c r="C7" s="3">
         <v>95</v>
       </c>
-      <c r="D7" s="3">
+      <c r="D7" s="7">
         <v>0.2677657000022009</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="F7" s="3">
+      <c r="F7" s="7">
         <v>0.24551729997619989</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="H7" s="3">
+      <c r="H7" s="7">
         <v>0.46548949996940792</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="J7" s="3">
+      <c r="J7" s="7">
         <v>0.39034099993295968</v>
       </c>
       <c r="K7" s="2" t="s">
@@ -1488,78 +1488,78 @@
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A8" s="11"/>
-      <c r="B8" s="11"/>
-      <c r="C8" s="8">
+      <c r="A8" s="10"/>
+      <c r="B8" s="10"/>
+      <c r="C8" s="3">
         <v>100</v>
       </c>
-      <c r="D8" s="3"/>
+      <c r="D8" s="7"/>
       <c r="E8" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="F8" s="3"/>
+      <c r="F8" s="7"/>
       <c r="G8" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="H8" s="3"/>
+      <c r="H8" s="7"/>
       <c r="I8" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="J8" s="3"/>
+      <c r="J8" s="7"/>
       <c r="K8" s="2" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A9" s="11"/>
-      <c r="B9" s="12"/>
-      <c r="C9" s="8">
+      <c r="A9" s="10"/>
+      <c r="B9" s="11"/>
+      <c r="C9" s="3">
         <v>105</v>
       </c>
-      <c r="D9" s="3"/>
+      <c r="D9" s="7"/>
       <c r="E9" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="F9" s="3"/>
+      <c r="F9" s="7"/>
       <c r="G9" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="H9" s="3"/>
+      <c r="H9" s="7"/>
       <c r="I9" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="J9" s="3"/>
+      <c r="J9" s="7"/>
       <c r="K9" s="2" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A10" s="11"/>
+      <c r="A10" s="10"/>
       <c r="B10" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C10" s="8">
+      <c r="C10" s="3">
         <v>95</v>
       </c>
-      <c r="D10" s="3">
+      <c r="D10" s="7">
         <v>1.5047430000267921</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="F10" s="3">
+      <c r="F10" s="7">
         <v>1.963980600005016</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="H10" s="3">
+      <c r="H10" s="7">
         <v>2.9798647999996319</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="J10" s="3">
+      <c r="J10" s="7">
         <v>3.39737579994835</v>
       </c>
       <c r="K10" s="2" t="s">
@@ -1567,78 +1567,78 @@
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A11" s="11"/>
-      <c r="B11" s="11"/>
-      <c r="C11" s="8">
+      <c r="A11" s="10"/>
+      <c r="B11" s="10"/>
+      <c r="C11" s="3">
         <v>100</v>
       </c>
-      <c r="D11" s="3"/>
+      <c r="D11" s="7"/>
       <c r="E11" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="F11" s="3"/>
+      <c r="F11" s="7"/>
       <c r="G11" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="H11" s="3"/>
+      <c r="H11" s="7"/>
       <c r="I11" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="J11" s="3"/>
+      <c r="J11" s="7"/>
       <c r="K11" s="2" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A12" s="11"/>
-      <c r="B12" s="12"/>
-      <c r="C12" s="8">
+      <c r="A12" s="10"/>
+      <c r="B12" s="11"/>
+      <c r="C12" s="3">
         <v>105</v>
       </c>
-      <c r="D12" s="3"/>
+      <c r="D12" s="7"/>
       <c r="E12" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="F12" s="3"/>
+      <c r="F12" s="7"/>
       <c r="G12" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="H12" s="3"/>
+      <c r="H12" s="7"/>
       <c r="I12" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="J12" s="3"/>
+      <c r="J12" s="7"/>
       <c r="K12" s="2" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A13" s="11"/>
+      <c r="A13" s="10"/>
       <c r="B13" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="C13" s="8">
+      <c r="C13" s="3">
         <v>95</v>
       </c>
-      <c r="D13" s="3">
+      <c r="D13" s="7">
         <v>14.52534100005869</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="F13" s="3">
+      <c r="F13" s="7">
         <v>20.233092900016349</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="H13" s="3">
+      <c r="H13" s="7">
         <v>29.562941399984989</v>
       </c>
       <c r="I13" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="J13" s="3">
+      <c r="J13" s="7">
         <v>48.585087500046939</v>
       </c>
       <c r="K13" s="2" t="s">
@@ -1646,47 +1646,47 @@
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A14" s="11"/>
-      <c r="B14" s="11"/>
-      <c r="C14" s="8">
+      <c r="A14" s="10"/>
+      <c r="B14" s="10"/>
+      <c r="C14" s="3">
         <v>100</v>
       </c>
-      <c r="D14" s="3"/>
+      <c r="D14" s="7"/>
       <c r="E14" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="F14" s="3"/>
+      <c r="F14" s="7"/>
       <c r="G14" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="H14" s="3"/>
+      <c r="H14" s="7"/>
       <c r="I14" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="J14" s="3"/>
+      <c r="J14" s="7"/>
       <c r="K14" s="2" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A15" s="12"/>
-      <c r="B15" s="12"/>
-      <c r="C15" s="8">
+      <c r="A15" s="11"/>
+      <c r="B15" s="11"/>
+      <c r="C15" s="3">
         <v>105</v>
       </c>
-      <c r="D15" s="3"/>
+      <c r="D15" s="7"/>
       <c r="E15" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="F15" s="3"/>
+      <c r="F15" s="7"/>
       <c r="G15" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="H15" s="3"/>
+      <c r="H15" s="7"/>
       <c r="I15" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="J15" s="3"/>
+      <c r="J15" s="7"/>
       <c r="K15" s="2" t="s">
         <v>61</v>
       </c>
@@ -1698,28 +1698,28 @@
       <c r="B16" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="C16" s="8">
+      <c r="C16" s="3">
         <v>95</v>
       </c>
-      <c r="D16" s="3">
+      <c r="D16" s="7">
         <v>0.238945999997668</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="F16" s="3">
+      <c r="F16" s="7">
         <v>0.24176189990248531</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="H16" s="3">
+      <c r="H16" s="7">
         <v>0.3870247999439016</v>
       </c>
       <c r="I16" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="J16" s="3">
+      <c r="J16" s="7">
         <v>0.44235779996961361</v>
       </c>
       <c r="K16" s="2" t="s">
@@ -1727,78 +1727,78 @@
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A17" s="11"/>
-      <c r="B17" s="11"/>
-      <c r="C17" s="8">
+      <c r="A17" s="10"/>
+      <c r="B17" s="10"/>
+      <c r="C17" s="3">
         <v>100</v>
       </c>
-      <c r="D17" s="3"/>
+      <c r="D17" s="7"/>
       <c r="E17" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="F17" s="3"/>
+      <c r="F17" s="7"/>
       <c r="G17" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="H17" s="3"/>
+      <c r="H17" s="7"/>
       <c r="I17" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="J17" s="3"/>
+      <c r="J17" s="7"/>
       <c r="K17" s="2" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A18" s="11"/>
-      <c r="B18" s="12"/>
-      <c r="C18" s="8">
+      <c r="A18" s="10"/>
+      <c r="B18" s="11"/>
+      <c r="C18" s="3">
         <v>105</v>
       </c>
-      <c r="D18" s="3"/>
+      <c r="D18" s="7"/>
       <c r="E18" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="F18" s="3"/>
+      <c r="F18" s="7"/>
       <c r="G18" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="H18" s="3"/>
+      <c r="H18" s="7"/>
       <c r="I18" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="J18" s="3"/>
+      <c r="J18" s="7"/>
       <c r="K18" s="2" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A19" s="11"/>
+      <c r="A19" s="10"/>
       <c r="B19" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C19" s="8">
+      <c r="C19" s="3">
         <v>95</v>
       </c>
-      <c r="D19" s="3">
+      <c r="D19" s="7">
         <v>1.4755197999766101</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="F19" s="3">
+      <c r="F19" s="7">
         <v>1.9966578999301421</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="H19" s="3">
+      <c r="H19" s="7">
         <v>2.863436799962074</v>
       </c>
       <c r="I19" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="J19" s="3">
+      <c r="J19" s="7">
         <v>3.373646300053224</v>
       </c>
       <c r="K19" s="2" t="s">
@@ -1806,78 +1806,78 @@
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A20" s="11"/>
-      <c r="B20" s="11"/>
-      <c r="C20" s="8">
+      <c r="A20" s="10"/>
+      <c r="B20" s="10"/>
+      <c r="C20" s="3">
         <v>100</v>
       </c>
-      <c r="D20" s="3"/>
+      <c r="D20" s="7"/>
       <c r="E20" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="F20" s="3"/>
+      <c r="F20" s="7"/>
       <c r="G20" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="H20" s="3"/>
+      <c r="H20" s="7"/>
       <c r="I20" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="J20" s="3"/>
+      <c r="J20" s="7"/>
       <c r="K20" s="2" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A21" s="11"/>
-      <c r="B21" s="12"/>
-      <c r="C21" s="8">
+      <c r="A21" s="10"/>
+      <c r="B21" s="11"/>
+      <c r="C21" s="3">
         <v>105</v>
       </c>
-      <c r="D21" s="3"/>
+      <c r="D21" s="7"/>
       <c r="E21" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="F21" s="3"/>
+      <c r="F21" s="7"/>
       <c r="G21" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="H21" s="3"/>
+      <c r="H21" s="7"/>
       <c r="I21" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="J21" s="3"/>
+      <c r="J21" s="7"/>
       <c r="K21" s="2" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A22" s="11"/>
+      <c r="A22" s="10"/>
       <c r="B22" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="C22" s="8">
+      <c r="C22" s="3">
         <v>95</v>
       </c>
-      <c r="D22" s="3">
+      <c r="D22" s="7">
         <v>14.46036919998005</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="F22" s="3">
+      <c r="F22" s="7">
         <v>19.967838000040501</v>
       </c>
       <c r="G22" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="H22" s="3">
+      <c r="H22" s="7">
         <v>28.54840089997742</v>
       </c>
       <c r="I22" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="J22" s="3">
+      <c r="J22" s="7">
         <v>48.517248400021337</v>
       </c>
       <c r="K22" s="2" t="s">
@@ -1885,47 +1885,47 @@
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A23" s="11"/>
-      <c r="B23" s="11"/>
-      <c r="C23" s="8">
+      <c r="A23" s="10"/>
+      <c r="B23" s="10"/>
+      <c r="C23" s="3">
         <v>100</v>
       </c>
-      <c r="D23" s="3"/>
+      <c r="D23" s="7"/>
       <c r="E23" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="F23" s="3"/>
+      <c r="F23" s="7"/>
       <c r="G23" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="H23" s="3"/>
+      <c r="H23" s="7"/>
       <c r="I23" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="J23" s="3"/>
+      <c r="J23" s="7"/>
       <c r="K23" s="2" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A24" s="12"/>
-      <c r="B24" s="12"/>
-      <c r="C24" s="8">
+      <c r="A24" s="11"/>
+      <c r="B24" s="11"/>
+      <c r="C24" s="3">
         <v>105</v>
       </c>
-      <c r="D24" s="3"/>
+      <c r="D24" s="7"/>
       <c r="E24" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="F24" s="3"/>
+      <c r="F24" s="7"/>
       <c r="G24" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="H24" s="3"/>
+      <c r="H24" s="7"/>
       <c r="I24" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="J24" s="3"/>
+      <c r="J24" s="7"/>
       <c r="K24" s="2" t="s">
         <v>97</v>
       </c>
@@ -1937,28 +1937,28 @@
       <c r="B25" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="C25" s="8">
+      <c r="C25" s="3">
         <v>47</v>
       </c>
-      <c r="D25" s="3">
+      <c r="D25" s="7">
         <v>8.9171500061638653E-2</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="F25" s="3">
+      <c r="F25" s="7">
         <v>8.3611599984578788E-2</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="H25" s="3">
+      <c r="H25" s="7">
         <v>0.10615459992550309</v>
       </c>
       <c r="I25" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="J25" s="3">
+      <c r="J25" s="7">
         <v>0.14980510005261749</v>
       </c>
       <c r="K25" s="2" t="s">
@@ -1966,124 +1966,124 @@
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A26" s="11"/>
-      <c r="B26" s="11"/>
-      <c r="C26" s="8">
+      <c r="A26" s="10"/>
+      <c r="B26" s="10"/>
+      <c r="C26" s="3">
         <v>48</v>
       </c>
-      <c r="D26" s="3"/>
+      <c r="D26" s="7"/>
       <c r="E26" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="F26" s="3"/>
+      <c r="F26" s="7"/>
       <c r="G26" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="H26" s="3"/>
+      <c r="H26" s="7"/>
       <c r="I26" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="J26" s="3"/>
+      <c r="J26" s="7"/>
       <c r="K26" s="2" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A27" s="11"/>
-      <c r="B27" s="11"/>
-      <c r="C27" s="8">
+      <c r="A27" s="10"/>
+      <c r="B27" s="10"/>
+      <c r="C27" s="3">
         <v>49</v>
       </c>
-      <c r="D27" s="3"/>
+      <c r="D27" s="7"/>
       <c r="E27" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="F27" s="3"/>
+      <c r="F27" s="7"/>
       <c r="G27" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="H27" s="3"/>
+      <c r="H27" s="7"/>
       <c r="I27" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="J27" s="3"/>
+      <c r="J27" s="7"/>
       <c r="K27" s="2" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A28" s="11"/>
-      <c r="B28" s="11"/>
-      <c r="C28" s="8">
+      <c r="A28" s="10"/>
+      <c r="B28" s="10"/>
+      <c r="C28" s="3">
         <v>50</v>
       </c>
-      <c r="D28" s="3"/>
+      <c r="D28" s="7"/>
       <c r="E28" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="F28" s="3"/>
+      <c r="F28" s="7"/>
       <c r="G28" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="H28" s="3"/>
+      <c r="H28" s="7"/>
       <c r="I28" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="J28" s="3"/>
+      <c r="J28" s="7"/>
       <c r="K28" s="2" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A29" s="11"/>
-      <c r="B29" s="12"/>
-      <c r="C29" s="8">
+      <c r="A29" s="10"/>
+      <c r="B29" s="11"/>
+      <c r="C29" s="3">
         <v>51</v>
       </c>
-      <c r="D29" s="3"/>
+      <c r="D29" s="7"/>
       <c r="E29" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="F29" s="3"/>
+      <c r="F29" s="7"/>
       <c r="G29" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="H29" s="3"/>
+      <c r="H29" s="7"/>
       <c r="I29" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="J29" s="3"/>
+      <c r="J29" s="7"/>
       <c r="K29" s="2" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A30" s="11"/>
+      <c r="A30" s="10"/>
       <c r="B30" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C30" s="8">
+      <c r="C30" s="3">
         <v>47</v>
       </c>
-      <c r="D30" s="3">
+      <c r="D30" s="7">
         <v>0.32301799999549979</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="F30" s="3">
+      <c r="F30" s="7">
         <v>0.43606109998654569</v>
       </c>
       <c r="G30" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="H30" s="3">
+      <c r="H30" s="7">
         <v>0.60521419998258352</v>
       </c>
       <c r="I30" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="J30" s="3">
+      <c r="J30" s="7">
         <v>0.70288489991798997</v>
       </c>
       <c r="K30" s="2" t="s">
@@ -2091,124 +2091,124 @@
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A31" s="11"/>
-      <c r="B31" s="11"/>
-      <c r="C31" s="8">
+      <c r="A31" s="10"/>
+      <c r="B31" s="10"/>
+      <c r="C31" s="3">
         <v>48</v>
       </c>
-      <c r="D31" s="3"/>
+      <c r="D31" s="7"/>
       <c r="E31" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="F31" s="3"/>
+      <c r="F31" s="7"/>
       <c r="G31" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="H31" s="3"/>
+      <c r="H31" s="7"/>
       <c r="I31" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="J31" s="3"/>
+      <c r="J31" s="7"/>
       <c r="K31" s="2" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A32" s="11"/>
-      <c r="B32" s="11"/>
-      <c r="C32" s="8">
+      <c r="A32" s="10"/>
+      <c r="B32" s="10"/>
+      <c r="C32" s="3">
         <v>49</v>
       </c>
-      <c r="D32" s="3"/>
+      <c r="D32" s="7"/>
       <c r="E32" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="F32" s="3"/>
+      <c r="F32" s="7"/>
       <c r="G32" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="H32" s="3"/>
+      <c r="H32" s="7"/>
       <c r="I32" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="J32" s="3"/>
+      <c r="J32" s="7"/>
       <c r="K32" s="2" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A33" s="11"/>
-      <c r="B33" s="11"/>
-      <c r="C33" s="8">
+      <c r="A33" s="10"/>
+      <c r="B33" s="10"/>
+      <c r="C33" s="3">
         <v>50</v>
       </c>
-      <c r="D33" s="3"/>
+      <c r="D33" s="7"/>
       <c r="E33" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="F33" s="3"/>
+      <c r="F33" s="7"/>
       <c r="G33" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="H33" s="3"/>
+      <c r="H33" s="7"/>
       <c r="I33" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="J33" s="3"/>
+      <c r="J33" s="7"/>
       <c r="K33" s="2" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A34" s="11"/>
-      <c r="B34" s="12"/>
-      <c r="C34" s="8">
+      <c r="A34" s="10"/>
+      <c r="B34" s="11"/>
+      <c r="C34" s="3">
         <v>51</v>
       </c>
-      <c r="D34" s="3"/>
+      <c r="D34" s="7"/>
       <c r="E34" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="F34" s="3"/>
+      <c r="F34" s="7"/>
       <c r="G34" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="H34" s="3"/>
+      <c r="H34" s="7"/>
       <c r="I34" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="J34" s="3"/>
+      <c r="J34" s="7"/>
       <c r="K34" s="2" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A35" s="11"/>
+      <c r="A35" s="10"/>
       <c r="B35" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="C35" s="8">
+      <c r="C35" s="3">
         <v>47</v>
       </c>
-      <c r="D35" s="3">
+      <c r="D35" s="7">
         <v>3.001315100002103</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="F35" s="3">
+      <c r="F35" s="7">
         <v>4.0081003999803224</v>
       </c>
       <c r="G35" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="H35" s="3">
+      <c r="H35" s="7">
         <v>5.7636176000814876</v>
       </c>
       <c r="I35" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="J35" s="3">
+      <c r="J35" s="7">
         <v>10.02923349989578</v>
       </c>
       <c r="K35" s="2" t="s">
@@ -2216,126 +2216,126 @@
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A36" s="11"/>
-      <c r="B36" s="11"/>
-      <c r="C36" s="8">
+      <c r="A36" s="10"/>
+      <c r="B36" s="10"/>
+      <c r="C36" s="3">
         <v>48</v>
       </c>
-      <c r="D36" s="3"/>
+      <c r="D36" s="7"/>
       <c r="E36" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="F36" s="3"/>
+      <c r="F36" s="7"/>
       <c r="G36" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="H36" s="3"/>
+      <c r="H36" s="7"/>
       <c r="I36" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="J36" s="3"/>
+      <c r="J36" s="7"/>
       <c r="K36" s="2" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A37" s="11"/>
-      <c r="B37" s="11"/>
-      <c r="C37" s="8">
+      <c r="A37" s="10"/>
+      <c r="B37" s="10"/>
+      <c r="C37" s="3">
         <v>49</v>
       </c>
-      <c r="D37" s="3"/>
+      <c r="D37" s="7"/>
       <c r="E37" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="F37" s="3"/>
+      <c r="F37" s="7"/>
       <c r="G37" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="H37" s="3"/>
+      <c r="H37" s="7"/>
       <c r="I37" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="J37" s="3"/>
+      <c r="J37" s="7"/>
       <c r="K37" s="2" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A38" s="11"/>
-      <c r="B38" s="11"/>
-      <c r="C38" s="8">
+      <c r="A38" s="10"/>
+      <c r="B38" s="10"/>
+      <c r="C38" s="3">
         <v>50</v>
       </c>
-      <c r="D38" s="3"/>
+      <c r="D38" s="7"/>
       <c r="E38" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="F38" s="3"/>
+      <c r="F38" s="7"/>
       <c r="G38" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="H38" s="3"/>
+      <c r="H38" s="7"/>
       <c r="I38" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="J38" s="3"/>
+      <c r="J38" s="7"/>
       <c r="K38" s="2" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A39" s="12"/>
-      <c r="B39" s="12"/>
-      <c r="C39" s="8">
+      <c r="A39" s="11"/>
+      <c r="B39" s="11"/>
+      <c r="C39" s="3">
         <v>51</v>
       </c>
-      <c r="D39" s="3"/>
+      <c r="D39" s="7"/>
       <c r="E39" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="F39" s="3"/>
+      <c r="F39" s="7"/>
       <c r="G39" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="H39" s="3"/>
+      <c r="H39" s="7"/>
       <c r="I39" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="J39" s="3"/>
+      <c r="J39" s="7"/>
       <c r="K39" s="2" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A40" s="5" t="s">
+      <c r="A40" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="B40" s="5" t="s">
+      <c r="B40" s="4" t="s">
         <v>10</v>
       </c>
       <c r="C40" s="1">
         <v>10</v>
       </c>
-      <c r="D40" s="3">
+      <c r="D40" s="7">
         <v>8.7301699910312891E-2</v>
       </c>
       <c r="E40" t="s">
         <v>160</v>
       </c>
-      <c r="F40" s="3">
+      <c r="F40" s="7">
         <v>8.4547300008125603E-2</v>
       </c>
       <c r="G40" t="s">
         <v>161</v>
       </c>
-      <c r="H40" s="3">
+      <c r="H40" s="7">
         <v>0.1103219001088291</v>
       </c>
       <c r="I40" t="s">
         <v>162</v>
       </c>
-      <c r="J40" s="3">
+      <c r="J40" s="7">
         <v>0.12990299996454269</v>
       </c>
       <c r="K40" t="s">
@@ -2343,78 +2343,78 @@
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A41" s="6"/>
-      <c r="B41" s="6"/>
+      <c r="A41" s="5"/>
+      <c r="B41" s="5"/>
       <c r="C41" s="1">
         <v>20</v>
       </c>
-      <c r="D41" s="4"/>
+      <c r="D41" s="8"/>
       <c r="E41" t="s">
         <v>164</v>
       </c>
-      <c r="F41" s="4"/>
+      <c r="F41" s="8"/>
       <c r="G41" t="s">
         <v>165</v>
       </c>
-      <c r="H41" s="4"/>
+      <c r="H41" s="8"/>
       <c r="I41" t="s">
         <v>166</v>
       </c>
-      <c r="J41" s="4"/>
+      <c r="J41" s="8"/>
       <c r="K41" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A42" s="6"/>
-      <c r="B42" s="7"/>
+      <c r="A42" s="5"/>
+      <c r="B42" s="6"/>
       <c r="C42" s="1">
         <v>40</v>
       </c>
-      <c r="D42" s="4"/>
+      <c r="D42" s="8"/>
       <c r="E42" t="s">
         <v>168</v>
       </c>
-      <c r="F42" s="4"/>
+      <c r="F42" s="8"/>
       <c r="G42" t="s">
         <v>169</v>
       </c>
-      <c r="H42" s="4"/>
+      <c r="H42" s="8"/>
       <c r="I42" t="s">
         <v>170</v>
       </c>
-      <c r="J42" s="4"/>
+      <c r="J42" s="8"/>
       <c r="K42" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A43" s="6"/>
-      <c r="B43" s="5" t="s">
+      <c r="A43" s="5"/>
+      <c r="B43" s="4" t="s">
         <v>15</v>
       </c>
       <c r="C43" s="1">
         <v>10</v>
       </c>
-      <c r="D43" s="3">
+      <c r="D43" s="7">
         <v>0.329887600033544</v>
       </c>
       <c r="E43" t="s">
         <v>172</v>
       </c>
-      <c r="F43" s="3">
+      <c r="F43" s="7">
         <v>0.42904950003139669</v>
       </c>
       <c r="G43" t="s">
         <v>173</v>
       </c>
-      <c r="H43" s="3">
+      <c r="H43" s="7">
         <v>0.58943910000380129</v>
       </c>
       <c r="I43" t="s">
         <v>174</v>
       </c>
-      <c r="J43" s="3">
+      <c r="J43" s="7">
         <v>0.70071749994531274</v>
       </c>
       <c r="K43" t="s">
@@ -2422,78 +2422,78 @@
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A44" s="6"/>
-      <c r="B44" s="6"/>
+      <c r="A44" s="5"/>
+      <c r="B44" s="5"/>
       <c r="C44" s="1">
         <v>20</v>
       </c>
-      <c r="D44" s="4"/>
+      <c r="D44" s="8"/>
       <c r="E44" t="s">
         <v>176</v>
       </c>
-      <c r="F44" s="4"/>
+      <c r="F44" s="8"/>
       <c r="G44" t="s">
         <v>177</v>
       </c>
-      <c r="H44" s="4"/>
+      <c r="H44" s="8"/>
       <c r="I44" t="s">
         <v>178</v>
       </c>
-      <c r="J44" s="4"/>
+      <c r="J44" s="8"/>
       <c r="K44" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A45" s="6"/>
-      <c r="B45" s="7"/>
+      <c r="A45" s="5"/>
+      <c r="B45" s="6"/>
       <c r="C45" s="1">
         <v>40</v>
       </c>
-      <c r="D45" s="4"/>
+      <c r="D45" s="8"/>
       <c r="E45" t="s">
         <v>180</v>
       </c>
-      <c r="F45" s="4"/>
+      <c r="F45" s="8"/>
       <c r="G45" t="s">
         <v>181</v>
       </c>
-      <c r="H45" s="4"/>
+      <c r="H45" s="8"/>
       <c r="I45" t="s">
         <v>182</v>
       </c>
-      <c r="J45" s="4"/>
+      <c r="J45" s="8"/>
       <c r="K45" t="s">
         <v>183</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A46" s="6"/>
-      <c r="B46" s="5" t="s">
+      <c r="A46" s="5"/>
+      <c r="B46" s="4" t="s">
         <v>20</v>
       </c>
       <c r="C46" s="1">
         <v>10</v>
       </c>
-      <c r="D46" s="3">
+      <c r="D46" s="7">
         <v>2.9262787998886779</v>
       </c>
       <c r="E46" t="s">
         <v>184</v>
       </c>
-      <c r="F46" s="3">
+      <c r="F46" s="7">
         <v>4.0733267000177884</v>
       </c>
       <c r="G46" t="s">
         <v>185</v>
       </c>
-      <c r="H46" s="3">
+      <c r="H46" s="7">
         <v>5.720168299973011</v>
       </c>
       <c r="I46" t="s">
         <v>186</v>
       </c>
-      <c r="J46" s="3">
+      <c r="J46" s="7">
         <v>9.9833600999554619</v>
       </c>
       <c r="K46" t="s">
@@ -2501,80 +2501,80 @@
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A47" s="6"/>
-      <c r="B47" s="6"/>
+      <c r="A47" s="5"/>
+      <c r="B47" s="5"/>
       <c r="C47" s="1">
         <v>20</v>
       </c>
-      <c r="D47" s="4"/>
+      <c r="D47" s="8"/>
       <c r="E47" t="s">
         <v>188</v>
       </c>
-      <c r="F47" s="4"/>
+      <c r="F47" s="8"/>
       <c r="G47" t="s">
         <v>189</v>
       </c>
-      <c r="H47" s="4"/>
+      <c r="H47" s="8"/>
       <c r="I47" t="s">
         <v>190</v>
       </c>
-      <c r="J47" s="4"/>
+      <c r="J47" s="8"/>
       <c r="K47" t="s">
         <v>191</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A48" s="7"/>
-      <c r="B48" s="7"/>
+      <c r="A48" s="6"/>
+      <c r="B48" s="6"/>
       <c r="C48" s="1">
         <v>40</v>
       </c>
-      <c r="D48" s="4"/>
+      <c r="D48" s="8"/>
       <c r="E48" t="s">
         <v>192</v>
       </c>
-      <c r="F48" s="4"/>
+      <c r="F48" s="8"/>
       <c r="G48" t="s">
         <v>193</v>
       </c>
-      <c r="H48" s="4"/>
+      <c r="H48" s="8"/>
       <c r="I48" t="s">
         <v>194</v>
       </c>
-      <c r="J48" s="4"/>
+      <c r="J48" s="8"/>
       <c r="K48" t="s">
         <v>195</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A49" s="5" t="s">
+      <c r="A49" s="4" t="s">
         <v>270</v>
       </c>
-      <c r="B49" s="5" t="s">
+      <c r="B49" s="4" t="s">
         <v>10</v>
       </c>
       <c r="C49" s="1">
         <v>47</v>
       </c>
-      <c r="D49" s="3">
+      <c r="D49" s="7">
         <v>0.38312290003523231</v>
       </c>
       <c r="E49" t="s">
         <v>196</v>
       </c>
-      <c r="F49" s="3">
+      <c r="F49" s="7">
         <v>0.43022370000835508</v>
       </c>
       <c r="G49" t="s">
         <v>197</v>
       </c>
-      <c r="H49" s="3">
+      <c r="H49" s="7">
         <v>0.78730580001138151</v>
       </c>
       <c r="I49" t="s">
         <v>198</v>
       </c>
-      <c r="J49" s="3">
+      <c r="J49" s="7">
         <v>0.70451229996979237</v>
       </c>
       <c r="K49" t="s">
@@ -2582,124 +2582,124 @@
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A50" s="6"/>
-      <c r="B50" s="6"/>
+      <c r="A50" s="5"/>
+      <c r="B50" s="5"/>
       <c r="C50" s="1">
         <v>48</v>
       </c>
-      <c r="D50" s="4"/>
+      <c r="D50" s="8"/>
       <c r="E50" t="s">
         <v>196</v>
       </c>
-      <c r="F50" s="4"/>
+      <c r="F50" s="8"/>
       <c r="G50" t="s">
         <v>199</v>
       </c>
-      <c r="H50" s="4"/>
+      <c r="H50" s="8"/>
       <c r="I50" t="s">
         <v>200</v>
       </c>
-      <c r="J50" s="4"/>
+      <c r="J50" s="8"/>
       <c r="K50" t="s">
         <v>196</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A51" s="6"/>
-      <c r="B51" s="6"/>
+      <c r="A51" s="5"/>
+      <c r="B51" s="5"/>
       <c r="C51" s="1">
         <v>49</v>
       </c>
-      <c r="D51" s="4"/>
+      <c r="D51" s="8"/>
       <c r="E51" t="s">
         <v>196</v>
       </c>
-      <c r="F51" s="4"/>
+      <c r="F51" s="8"/>
       <c r="G51" t="s">
         <v>201</v>
       </c>
-      <c r="H51" s="4"/>
+      <c r="H51" s="8"/>
       <c r="I51" t="s">
         <v>202</v>
       </c>
-      <c r="J51" s="4"/>
+      <c r="J51" s="8"/>
       <c r="K51" t="s">
         <v>196</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A52" s="6"/>
-      <c r="B52" s="6"/>
+      <c r="A52" s="5"/>
+      <c r="B52" s="5"/>
       <c r="C52" s="1">
         <v>50</v>
       </c>
-      <c r="D52" s="4"/>
+      <c r="D52" s="8"/>
       <c r="E52" t="s">
         <v>196</v>
       </c>
-      <c r="F52" s="4"/>
+      <c r="F52" s="8"/>
       <c r="G52" t="s">
         <v>203</v>
       </c>
-      <c r="H52" s="4"/>
+      <c r="H52" s="8"/>
       <c r="I52" t="s">
         <v>204</v>
       </c>
-      <c r="J52" s="4"/>
+      <c r="J52" s="8"/>
       <c r="K52" t="s">
         <v>196</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A53" s="6"/>
-      <c r="B53" s="7"/>
+      <c r="A53" s="5"/>
+      <c r="B53" s="6"/>
       <c r="C53" s="1">
         <v>51</v>
       </c>
-      <c r="D53" s="4"/>
+      <c r="D53" s="8"/>
       <c r="E53" t="s">
         <v>196</v>
       </c>
-      <c r="F53" s="4"/>
+      <c r="F53" s="8"/>
       <c r="G53" t="s">
         <v>205</v>
       </c>
-      <c r="H53" s="4"/>
+      <c r="H53" s="8"/>
       <c r="I53" t="s">
         <v>206</v>
       </c>
-      <c r="J53" s="4"/>
+      <c r="J53" s="8"/>
       <c r="K53" t="s">
         <v>196</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A54" s="6"/>
-      <c r="B54" s="5" t="s">
+      <c r="A54" s="5"/>
+      <c r="B54" s="4" t="s">
         <v>15</v>
       </c>
       <c r="C54" s="1">
         <v>47</v>
       </c>
-      <c r="D54" s="3">
+      <c r="D54" s="7">
         <v>2.8947976999916141</v>
       </c>
       <c r="E54" t="s">
         <v>196</v>
       </c>
-      <c r="F54" s="3">
+      <c r="F54" s="7">
         <v>3.8898246999597181</v>
       </c>
       <c r="G54" t="s">
         <v>207</v>
       </c>
-      <c r="H54" s="3">
+      <c r="H54" s="7">
         <v>5.8676512000383809</v>
       </c>
       <c r="I54" t="s">
         <v>208</v>
       </c>
-      <c r="J54" s="3">
+      <c r="J54" s="7">
         <v>6.6754493000917137</v>
       </c>
       <c r="K54" t="s">
@@ -2707,124 +2707,124 @@
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A55" s="6"/>
-      <c r="B55" s="6"/>
+      <c r="A55" s="5"/>
+      <c r="B55" s="5"/>
       <c r="C55" s="1">
         <v>48</v>
       </c>
-      <c r="D55" s="4"/>
+      <c r="D55" s="8"/>
       <c r="E55" t="s">
         <v>196</v>
       </c>
-      <c r="F55" s="4"/>
+      <c r="F55" s="8"/>
       <c r="G55" t="s">
         <v>210</v>
       </c>
-      <c r="H55" s="4"/>
+      <c r="H55" s="8"/>
       <c r="I55" t="s">
         <v>211</v>
       </c>
-      <c r="J55" s="4"/>
+      <c r="J55" s="8"/>
       <c r="K55" t="s">
         <v>209</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A56" s="6"/>
-      <c r="B56" s="6"/>
+      <c r="A56" s="5"/>
+      <c r="B56" s="5"/>
       <c r="C56" s="1">
         <v>49</v>
       </c>
-      <c r="D56" s="4"/>
+      <c r="D56" s="8"/>
       <c r="E56" t="s">
         <v>196</v>
       </c>
-      <c r="F56" s="4"/>
+      <c r="F56" s="8"/>
       <c r="G56" t="s">
         <v>212</v>
       </c>
-      <c r="H56" s="4"/>
+      <c r="H56" s="8"/>
       <c r="I56" t="s">
         <v>213</v>
       </c>
-      <c r="J56" s="4"/>
+      <c r="J56" s="8"/>
       <c r="K56" t="s">
         <v>209</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A57" s="6"/>
-      <c r="B57" s="6"/>
+      <c r="A57" s="5"/>
+      <c r="B57" s="5"/>
       <c r="C57" s="1">
         <v>50</v>
       </c>
-      <c r="D57" s="4"/>
+      <c r="D57" s="8"/>
       <c r="E57" t="s">
         <v>196</v>
       </c>
-      <c r="F57" s="4"/>
+      <c r="F57" s="8"/>
       <c r="G57" t="s">
         <v>214</v>
       </c>
-      <c r="H57" s="4"/>
+      <c r="H57" s="8"/>
       <c r="I57" t="s">
         <v>215</v>
       </c>
-      <c r="J57" s="4"/>
+      <c r="J57" s="8"/>
       <c r="K57" t="s">
         <v>209</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A58" s="6"/>
-      <c r="B58" s="7"/>
+      <c r="A58" s="5"/>
+      <c r="B58" s="6"/>
       <c r="C58" s="1">
         <v>51</v>
       </c>
-      <c r="D58" s="4"/>
+      <c r="D58" s="8"/>
       <c r="E58" t="s">
         <v>196</v>
       </c>
-      <c r="F58" s="4"/>
+      <c r="F58" s="8"/>
       <c r="G58" t="s">
         <v>216</v>
       </c>
-      <c r="H58" s="4"/>
+      <c r="H58" s="8"/>
       <c r="I58" t="s">
         <v>217</v>
       </c>
-      <c r="J58" s="4"/>
+      <c r="J58" s="8"/>
       <c r="K58" t="s">
         <v>209</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A59" s="6"/>
-      <c r="B59" s="5" t="s">
+      <c r="A59" s="5"/>
+      <c r="B59" s="4" t="s">
         <v>20</v>
       </c>
       <c r="C59" s="1">
         <v>47</v>
       </c>
-      <c r="D59" s="3">
+      <c r="D59" s="7">
         <v>29.223953899927441</v>
       </c>
       <c r="E59" t="s">
         <v>218</v>
       </c>
-      <c r="F59" s="3">
+      <c r="F59" s="7">
         <v>55.427861100062728</v>
       </c>
       <c r="G59" t="s">
         <v>219</v>
       </c>
-      <c r="H59" s="3">
+      <c r="H59" s="7">
         <v>57.770199500024319</v>
       </c>
       <c r="I59" t="s">
         <v>220</v>
       </c>
-      <c r="J59" s="3">
+      <c r="J59" s="7">
         <v>99.37938940001186</v>
       </c>
       <c r="K59" t="s">
@@ -2832,126 +2832,126 @@
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A60" s="6"/>
-      <c r="B60" s="6"/>
+      <c r="A60" s="5"/>
+      <c r="B60" s="5"/>
       <c r="C60" s="1">
         <v>48</v>
       </c>
-      <c r="D60" s="4"/>
+      <c r="D60" s="8"/>
       <c r="E60" t="s">
         <v>222</v>
       </c>
-      <c r="F60" s="4"/>
+      <c r="F60" s="8"/>
       <c r="G60" t="s">
         <v>223</v>
       </c>
-      <c r="H60" s="4"/>
+      <c r="H60" s="8"/>
       <c r="I60" t="s">
         <v>224</v>
       </c>
-      <c r="J60" s="4"/>
+      <c r="J60" s="8"/>
       <c r="K60" t="s">
         <v>221</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A61" s="6"/>
-      <c r="B61" s="6"/>
+      <c r="A61" s="5"/>
+      <c r="B61" s="5"/>
       <c r="C61" s="1">
         <v>49</v>
       </c>
-      <c r="D61" s="4"/>
+      <c r="D61" s="8"/>
       <c r="E61" t="s">
         <v>225</v>
       </c>
-      <c r="F61" s="4"/>
+      <c r="F61" s="8"/>
       <c r="G61" t="s">
         <v>226</v>
       </c>
-      <c r="H61" s="4"/>
+      <c r="H61" s="8"/>
       <c r="I61" t="s">
         <v>227</v>
       </c>
-      <c r="J61" s="4"/>
+      <c r="J61" s="8"/>
       <c r="K61" t="s">
         <v>221</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A62" s="6"/>
-      <c r="B62" s="6"/>
+      <c r="A62" s="5"/>
+      <c r="B62" s="5"/>
       <c r="C62" s="1">
         <v>50</v>
       </c>
-      <c r="D62" s="4"/>
+      <c r="D62" s="8"/>
       <c r="E62" t="s">
         <v>228</v>
       </c>
-      <c r="F62" s="4"/>
+      <c r="F62" s="8"/>
       <c r="G62" t="s">
         <v>229</v>
       </c>
-      <c r="H62" s="4"/>
+      <c r="H62" s="8"/>
       <c r="I62" t="s">
         <v>230</v>
       </c>
-      <c r="J62" s="4"/>
+      <c r="J62" s="8"/>
       <c r="K62" t="s">
         <v>221</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A63" s="7"/>
-      <c r="B63" s="7"/>
+      <c r="A63" s="6"/>
+      <c r="B63" s="6"/>
       <c r="C63" s="1">
         <v>51</v>
       </c>
-      <c r="D63" s="4"/>
+      <c r="D63" s="8"/>
       <c r="E63" t="s">
         <v>231</v>
       </c>
-      <c r="F63" s="4"/>
+      <c r="F63" s="8"/>
       <c r="G63" t="s">
         <v>232</v>
       </c>
-      <c r="H63" s="4"/>
+      <c r="H63" s="8"/>
       <c r="I63" t="s">
         <v>233</v>
       </c>
-      <c r="J63" s="4"/>
+      <c r="J63" s="8"/>
       <c r="K63" t="s">
         <v>221</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A64" s="5" t="s">
+      <c r="A64" s="4" t="s">
         <v>234</v>
       </c>
-      <c r="B64" s="5" t="s">
+      <c r="B64" s="4" t="s">
         <v>10</v>
       </c>
       <c r="C64" s="1">
         <v>95</v>
       </c>
-      <c r="D64" s="3">
+      <c r="D64" s="7">
         <v>0.21036979998461899</v>
       </c>
       <c r="E64" t="s">
         <v>235</v>
       </c>
-      <c r="F64" s="3">
+      <c r="F64" s="7">
         <v>0.24970609997399151</v>
       </c>
       <c r="G64" t="s">
         <v>236</v>
       </c>
-      <c r="H64" s="3">
+      <c r="H64" s="7">
         <v>0.37662180000916118</v>
       </c>
       <c r="I64" t="s">
         <v>237</v>
       </c>
-      <c r="J64" s="3">
+      <c r="J64" s="7">
         <v>0.37422160001005977</v>
       </c>
       <c r="K64" t="s">
@@ -2959,78 +2959,78 @@
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A65" s="6"/>
-      <c r="B65" s="6"/>
+      <c r="A65" s="5"/>
+      <c r="B65" s="5"/>
       <c r="C65" s="1">
         <v>100</v>
       </c>
-      <c r="D65" s="4"/>
+      <c r="D65" s="8"/>
       <c r="E65" t="s">
         <v>239</v>
       </c>
-      <c r="F65" s="4"/>
+      <c r="F65" s="8"/>
       <c r="G65" t="s">
         <v>240</v>
       </c>
-      <c r="H65" s="4"/>
+      <c r="H65" s="8"/>
       <c r="I65" t="s">
         <v>241</v>
       </c>
-      <c r="J65" s="4"/>
+      <c r="J65" s="8"/>
       <c r="K65" t="s">
         <v>242</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A66" s="6"/>
-      <c r="B66" s="7"/>
+      <c r="A66" s="5"/>
+      <c r="B66" s="6"/>
       <c r="C66" s="1">
         <v>105</v>
       </c>
-      <c r="D66" s="4"/>
+      <c r="D66" s="8"/>
       <c r="E66" t="s">
         <v>243</v>
       </c>
-      <c r="F66" s="4"/>
+      <c r="F66" s="8"/>
       <c r="G66" t="s">
         <v>244</v>
       </c>
-      <c r="H66" s="4"/>
+      <c r="H66" s="8"/>
       <c r="I66" t="s">
         <v>245</v>
       </c>
-      <c r="J66" s="4"/>
+      <c r="J66" s="8"/>
       <c r="K66" t="s">
         <v>246</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A67" s="6"/>
-      <c r="B67" s="5" t="s">
+      <c r="A67" s="5"/>
+      <c r="B67" s="4" t="s">
         <v>15</v>
       </c>
       <c r="C67" s="1">
         <v>95</v>
       </c>
-      <c r="D67" s="3">
+      <c r="D67" s="7">
         <v>1.4952732999809091</v>
       </c>
       <c r="E67" t="s">
         <v>247</v>
       </c>
-      <c r="F67" s="3">
+      <c r="F67" s="7">
         <v>1.938804800040089</v>
       </c>
       <c r="G67" t="s">
         <v>248</v>
       </c>
-      <c r="H67" s="3">
+      <c r="H67" s="7">
         <v>2.9082565000280738</v>
       </c>
       <c r="I67" t="s">
         <v>249</v>
       </c>
-      <c r="J67" s="3">
+      <c r="J67" s="7">
         <v>3.3668100000359118</v>
       </c>
       <c r="K67" t="s">
@@ -3038,78 +3038,78 @@
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A68" s="6"/>
-      <c r="B68" s="6"/>
+      <c r="A68" s="5"/>
+      <c r="B68" s="5"/>
       <c r="C68" s="1">
         <v>100</v>
       </c>
-      <c r="D68" s="4"/>
+      <c r="D68" s="8"/>
       <c r="E68" t="s">
         <v>251</v>
       </c>
-      <c r="F68" s="4"/>
+      <c r="F68" s="8"/>
       <c r="G68" t="s">
         <v>252</v>
       </c>
-      <c r="H68" s="4"/>
+      <c r="H68" s="8"/>
       <c r="I68" t="s">
         <v>253</v>
       </c>
-      <c r="J68" s="4"/>
+      <c r="J68" s="8"/>
       <c r="K68" t="s">
         <v>254</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A69" s="6"/>
-      <c r="B69" s="7"/>
+      <c r="A69" s="5"/>
+      <c r="B69" s="6"/>
       <c r="C69" s="1">
         <v>105</v>
       </c>
-      <c r="D69" s="4"/>
+      <c r="D69" s="8"/>
       <c r="E69" t="s">
         <v>255</v>
       </c>
-      <c r="F69" s="4"/>
+      <c r="F69" s="8"/>
       <c r="G69" t="s">
         <v>256</v>
       </c>
-      <c r="H69" s="4"/>
+      <c r="H69" s="8"/>
       <c r="I69" t="s">
         <v>257</v>
       </c>
-      <c r="J69" s="4"/>
+      <c r="J69" s="8"/>
       <c r="K69" t="s">
         <v>258</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A70" s="6"/>
-      <c r="B70" s="5" t="s">
+      <c r="A70" s="5"/>
+      <c r="B70" s="4" t="s">
         <v>20</v>
       </c>
       <c r="C70" s="1">
         <v>95</v>
       </c>
-      <c r="D70" s="3">
+      <c r="D70" s="7">
         <v>14.7206091999542</v>
       </c>
       <c r="E70" t="s">
         <v>259</v>
       </c>
-      <c r="F70" s="3">
+      <c r="F70" s="7">
         <v>34.249781799968332</v>
       </c>
       <c r="G70" t="s">
         <v>260</v>
       </c>
-      <c r="H70" s="3">
+      <c r="H70" s="7">
         <v>48.121484700008303</v>
       </c>
       <c r="I70" t="s">
         <v>261</v>
       </c>
-      <c r="J70" s="3">
+      <c r="J70" s="7">
         <v>52.205460399971336</v>
       </c>
       <c r="K70" t="s">
@@ -3117,98 +3117,77 @@
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A71" s="6"/>
-      <c r="B71" s="6"/>
+      <c r="A71" s="5"/>
+      <c r="B71" s="5"/>
       <c r="C71" s="1">
         <v>100</v>
       </c>
-      <c r="D71" s="4"/>
+      <c r="D71" s="8"/>
       <c r="E71" t="s">
         <v>262</v>
       </c>
-      <c r="F71" s="4"/>
+      <c r="F71" s="8"/>
       <c r="G71" t="s">
         <v>263</v>
       </c>
-      <c r="H71" s="4"/>
+      <c r="H71" s="8"/>
       <c r="I71" t="s">
         <v>264</v>
       </c>
-      <c r="J71" s="4"/>
+      <c r="J71" s="8"/>
       <c r="K71" t="s">
         <v>265</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A72" s="7"/>
-      <c r="B72" s="7"/>
+      <c r="A72" s="6"/>
+      <c r="B72" s="6"/>
       <c r="C72" s="1">
         <v>105</v>
       </c>
-      <c r="D72" s="4"/>
+      <c r="D72" s="8"/>
       <c r="E72" t="s">
         <v>266</v>
       </c>
-      <c r="F72" s="4"/>
+      <c r="F72" s="8"/>
       <c r="G72" t="s">
         <v>267</v>
       </c>
-      <c r="H72" s="4"/>
+      <c r="H72" s="8"/>
       <c r="I72" t="s">
         <v>268</v>
       </c>
-      <c r="J72" s="4"/>
+      <c r="J72" s="8"/>
       <c r="K72" t="s">
         <v>269</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="101">
-    <mergeCell ref="B67:B69"/>
-    <mergeCell ref="A49:A63"/>
-    <mergeCell ref="D64:D66"/>
-    <mergeCell ref="J22:J24"/>
-    <mergeCell ref="F64:F66"/>
-    <mergeCell ref="B30:B34"/>
-    <mergeCell ref="A25:A39"/>
-    <mergeCell ref="B64:B66"/>
-    <mergeCell ref="D30:D34"/>
-    <mergeCell ref="F10:F12"/>
-    <mergeCell ref="B54:B58"/>
-    <mergeCell ref="D54:D58"/>
-    <mergeCell ref="H30:H34"/>
-    <mergeCell ref="D40:D42"/>
-    <mergeCell ref="F40:F42"/>
-    <mergeCell ref="J13:J15"/>
-    <mergeCell ref="J64:J66"/>
-    <mergeCell ref="H43:H45"/>
-    <mergeCell ref="A40:A48"/>
-    <mergeCell ref="D49:D53"/>
-    <mergeCell ref="B13:B15"/>
-    <mergeCell ref="D13:D15"/>
-    <mergeCell ref="B19:B21"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="F22:F24"/>
-    <mergeCell ref="H22:H24"/>
-    <mergeCell ref="J35:J39"/>
-    <mergeCell ref="F46:F48"/>
-    <mergeCell ref="J25:J29"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="H16:H18"/>
-    <mergeCell ref="J16:J18"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="B49:B53"/>
-    <mergeCell ref="J43:J45"/>
-    <mergeCell ref="A4:A6"/>
-    <mergeCell ref="D19:D21"/>
-    <mergeCell ref="F19:F21"/>
-    <mergeCell ref="B35:B39"/>
-    <mergeCell ref="D35:D39"/>
-    <mergeCell ref="B25:B29"/>
-    <mergeCell ref="B46:B48"/>
-    <mergeCell ref="D46:D48"/>
-    <mergeCell ref="F30:F34"/>
-    <mergeCell ref="J30:J34"/>
+    <mergeCell ref="H70:H72"/>
+    <mergeCell ref="F35:F39"/>
+    <mergeCell ref="H19:H21"/>
+    <mergeCell ref="F49:F53"/>
+    <mergeCell ref="D25:D29"/>
+    <mergeCell ref="B7:B9"/>
+    <mergeCell ref="H67:H69"/>
+    <mergeCell ref="J67:J69"/>
+    <mergeCell ref="B59:B63"/>
+    <mergeCell ref="B22:B24"/>
+    <mergeCell ref="D59:D63"/>
+    <mergeCell ref="D22:D24"/>
+    <mergeCell ref="H35:H39"/>
+    <mergeCell ref="F25:F29"/>
+    <mergeCell ref="D67:D69"/>
+    <mergeCell ref="F67:F69"/>
+    <mergeCell ref="F54:F58"/>
+    <mergeCell ref="H54:H58"/>
+    <mergeCell ref="F16:F18"/>
+    <mergeCell ref="H10:H12"/>
+    <mergeCell ref="J10:J12"/>
+    <mergeCell ref="J19:J21"/>
+    <mergeCell ref="H49:H53"/>
+    <mergeCell ref="J49:J53"/>
     <mergeCell ref="D1:E1"/>
     <mergeCell ref="B40:B42"/>
     <mergeCell ref="J46:J48"/>
@@ -3233,38 +3212,59 @@
     <mergeCell ref="J70:J72"/>
     <mergeCell ref="F13:F15"/>
     <mergeCell ref="D43:D45"/>
+    <mergeCell ref="A4:A6"/>
+    <mergeCell ref="D19:D21"/>
+    <mergeCell ref="F19:F21"/>
+    <mergeCell ref="B35:B39"/>
+    <mergeCell ref="D35:D39"/>
+    <mergeCell ref="B25:B29"/>
+    <mergeCell ref="B46:B48"/>
+    <mergeCell ref="D46:D48"/>
+    <mergeCell ref="F30:F34"/>
+    <mergeCell ref="F43:F45"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="F22:F24"/>
+    <mergeCell ref="H22:H24"/>
+    <mergeCell ref="J35:J39"/>
+    <mergeCell ref="F46:F48"/>
+    <mergeCell ref="J25:J29"/>
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="H16:H18"/>
+    <mergeCell ref="J16:J18"/>
+    <mergeCell ref="J1:K1"/>
+    <mergeCell ref="J43:J45"/>
+    <mergeCell ref="J30:J34"/>
     <mergeCell ref="H7:H9"/>
     <mergeCell ref="J7:J9"/>
-    <mergeCell ref="F43:F45"/>
+    <mergeCell ref="H25:H29"/>
+    <mergeCell ref="F10:F12"/>
+    <mergeCell ref="B54:B58"/>
+    <mergeCell ref="D54:D58"/>
+    <mergeCell ref="H30:H34"/>
+    <mergeCell ref="D40:D42"/>
+    <mergeCell ref="F40:F42"/>
+    <mergeCell ref="J13:J15"/>
+    <mergeCell ref="J64:J66"/>
+    <mergeCell ref="H43:H45"/>
+    <mergeCell ref="D49:D53"/>
+    <mergeCell ref="B13:B15"/>
+    <mergeCell ref="D13:D15"/>
+    <mergeCell ref="B19:B21"/>
+    <mergeCell ref="B49:B53"/>
     <mergeCell ref="H64:H66"/>
     <mergeCell ref="F59:F63"/>
     <mergeCell ref="H59:H63"/>
     <mergeCell ref="J59:J63"/>
-    <mergeCell ref="H70:H72"/>
-    <mergeCell ref="F35:F39"/>
-    <mergeCell ref="H19:H21"/>
-    <mergeCell ref="F49:F53"/>
-    <mergeCell ref="D25:D29"/>
-    <mergeCell ref="B7:B9"/>
-    <mergeCell ref="H67:H69"/>
-    <mergeCell ref="J67:J69"/>
-    <mergeCell ref="B59:B63"/>
-    <mergeCell ref="B22:B24"/>
-    <mergeCell ref="D59:D63"/>
-    <mergeCell ref="D22:D24"/>
-    <mergeCell ref="H35:H39"/>
-    <mergeCell ref="F25:F29"/>
-    <mergeCell ref="D67:D69"/>
-    <mergeCell ref="F67:F69"/>
-    <mergeCell ref="F54:F58"/>
-    <mergeCell ref="H54:H58"/>
-    <mergeCell ref="F16:F18"/>
-    <mergeCell ref="H10:H12"/>
-    <mergeCell ref="J10:J12"/>
-    <mergeCell ref="J19:J21"/>
-    <mergeCell ref="H49:H53"/>
-    <mergeCell ref="J49:J53"/>
-    <mergeCell ref="H25:H29"/>
+    <mergeCell ref="B67:B69"/>
+    <mergeCell ref="A49:A63"/>
+    <mergeCell ref="D64:D66"/>
+    <mergeCell ref="J22:J24"/>
+    <mergeCell ref="F64:F66"/>
+    <mergeCell ref="B30:B34"/>
+    <mergeCell ref="A25:A39"/>
+    <mergeCell ref="B64:B66"/>
+    <mergeCell ref="D30:D34"/>
+    <mergeCell ref="A40:A48"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>